<commit_message>
added connection to sql database
</commit_message>
<xml_diff>
--- a/unit_tests/test_cases.xlsx
+++ b/unit_tests/test_cases.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aa4f6975e0189fcb/Documents/Source/Cars/unit_tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="55" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{81AA0CED-5750-49A9-BCB4-E6B39777CF74}"/>
+  <xr:revisionPtr revIDLastSave="92" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9AB02D3A-DF3B-4706-9B5A-7CA059C1EA1C}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-2655" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{E1449062-40AE-488A-A0E8-5543147B756E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{E1449062-40AE-488A-A0E8-5543147B756E}"/>
   </bookViews>
   <sheets>
     <sheet name="TC-D5" sheetId="1" r:id="rId1"/>
     <sheet name="TC-D2-FG-D1" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
     <sheet name="Design" sheetId="5" r:id="rId4"/>
-    <sheet name="CoordinateDirection" sheetId="4" r:id="rId5"/>
+    <sheet name="Database-Design" sheetId="6" r:id="rId5"/>
+    <sheet name="CoordinateDirection" sheetId="4" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="66">
   <si>
     <t>Gallon per mile</t>
   </si>
@@ -178,6 +179,66 @@
   </si>
   <si>
     <t>AddBattery</t>
+  </si>
+  <si>
+    <t>Database</t>
+  </si>
+  <si>
+    <t>CarExplorer</t>
+  </si>
+  <si>
+    <t>Schema/Folder</t>
+  </si>
+  <si>
+    <t>game</t>
+  </si>
+  <si>
+    <t>component</t>
+  </si>
+  <si>
+    <t>factory</t>
+  </si>
+  <si>
+    <t>Table</t>
+  </si>
+  <si>
+    <t>CarID</t>
+  </si>
+  <si>
+    <t>Model</t>
+  </si>
+  <si>
+    <t>game.Cars</t>
+  </si>
+  <si>
+    <t>game.Trips</t>
+  </si>
+  <si>
+    <t>Make</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>TripID</t>
+  </si>
+  <si>
+    <t>StartX</t>
+  </si>
+  <si>
+    <t>StartY</t>
+  </si>
+  <si>
+    <t>EndX</t>
+  </si>
+  <si>
+    <t>EndY</t>
+  </si>
+  <si>
+    <t>StartDateTime</t>
+  </si>
+  <si>
+    <t>EndDateTime</t>
   </si>
 </sst>
 </file>
@@ -1442,6 +1503,95 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C68B0F5-EBBE-43FB-B76D-76A1F84FE911}">
+  <dimension ref="F1:O9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="6" max="6" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="6:15" x14ac:dyDescent="0.3">
+      <c r="F1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="6:15" x14ac:dyDescent="0.3">
+      <c r="F3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="6:15" x14ac:dyDescent="0.3">
+      <c r="G4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="6:15" x14ac:dyDescent="0.3">
+      <c r="G5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" spans="6:15" x14ac:dyDescent="0.3">
+      <c r="F8" t="s">
+        <v>52</v>
+      </c>
+      <c r="G8" t="s">
+        <v>55</v>
+      </c>
+      <c r="H8" t="s">
+        <v>53</v>
+      </c>
+      <c r="I8" t="s">
+        <v>57</v>
+      </c>
+      <c r="J8" t="s">
+        <v>54</v>
+      </c>
+      <c r="K8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" spans="6:15" x14ac:dyDescent="0.3">
+      <c r="G9" t="s">
+        <v>56</v>
+      </c>
+      <c r="H9" t="s">
+        <v>59</v>
+      </c>
+      <c r="I9" t="s">
+        <v>53</v>
+      </c>
+      <c r="J9" t="s">
+        <v>60</v>
+      </c>
+      <c r="K9" t="s">
+        <v>61</v>
+      </c>
+      <c r="L9" t="s">
+        <v>62</v>
+      </c>
+      <c r="M9" t="s">
+        <v>63</v>
+      </c>
+      <c r="N9" t="s">
+        <v>64</v>
+      </c>
+      <c r="O9" t="s">
+        <v>65</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1643BAB-DCF5-4FE9-88FC-DB471EA141B5}">
   <dimension ref="F10:L15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
Insert trip details to database
</commit_message>
<xml_diff>
--- a/unit_tests/test_cases.xlsx
+++ b/unit_tests/test_cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aa4f6975e0189fcb/Documents/Source/Cars/unit_tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="92" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9AB02D3A-DF3B-4706-9B5A-7CA059C1EA1C}"/>
+  <xr:revisionPtr revIDLastSave="109" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{630AFC59-4944-4545-A9A6-9EE4B8B1867D}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{E1449062-40AE-488A-A0E8-5543147B756E}"/>
+    <workbookView minimized="1" xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="8880" activeTab="4" xr2:uid="{E1449062-40AE-488A-A0E8-5543147B756E}"/>
   </bookViews>
   <sheets>
     <sheet name="TC-D5" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="75">
   <si>
     <t>Gallon per mile</t>
   </si>
@@ -239,6 +239,33 @@
   </si>
   <si>
     <t>EndDateTime</t>
+  </si>
+  <si>
+    <t>select top 5 * from cars</t>
+  </si>
+  <si>
+    <t>Get the first row from the result set</t>
+  </si>
+  <si>
+    <t>print the row out</t>
+  </si>
+  <si>
+    <t>Get the individual fields from the first row</t>
+  </si>
+  <si>
+    <t>assign to python variable, carid, make, model, year</t>
+  </si>
+  <si>
+    <t>Get the trips using the car id order by end time desc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assign to python variable, </t>
+  </si>
+  <si>
+    <t>Build the car using the fields above, car_a</t>
+  </si>
+  <si>
+    <t>Assign the car above with ending X and Y</t>
   </si>
 </sst>
 </file>
@@ -1504,7 +1531,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C68B0F5-EBBE-43FB-B76D-76A1F84FE911}">
-  <dimension ref="F1:O9"/>
+  <dimension ref="F1:P23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="6" max="6" width="13.44140625" bestFit="1" customWidth="1"/>
@@ -1584,6 +1611,82 @@
       </c>
       <c r="O9" t="s">
         <v>65</v>
+      </c>
+    </row>
+    <row r="12" spans="6:15" x14ac:dyDescent="0.3">
+      <c r="F12" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="13" spans="6:15" x14ac:dyDescent="0.3">
+      <c r="F13" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="14" spans="6:15" x14ac:dyDescent="0.3">
+      <c r="G14" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="15" spans="6:15" x14ac:dyDescent="0.3">
+      <c r="F15" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="16" spans="6:15" x14ac:dyDescent="0.3">
+      <c r="G16" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="17" spans="6:16" x14ac:dyDescent="0.3">
+      <c r="F17" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="19" spans="6:16" x14ac:dyDescent="0.3">
+      <c r="F19" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="20" spans="6:16" x14ac:dyDescent="0.3">
+      <c r="F20" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="21" spans="6:16" x14ac:dyDescent="0.3">
+      <c r="F21" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="22" spans="6:16" x14ac:dyDescent="0.3">
+      <c r="G22" t="s">
+        <v>72</v>
+      </c>
+      <c r="I22" t="s">
+        <v>59</v>
+      </c>
+      <c r="K22" t="s">
+        <v>60</v>
+      </c>
+      <c r="L22" t="s">
+        <v>61</v>
+      </c>
+      <c r="M22" t="s">
+        <v>62</v>
+      </c>
+      <c r="N22" t="s">
+        <v>63</v>
+      </c>
+      <c r="O22" t="s">
+        <v>64</v>
+      </c>
+      <c r="P22" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="23" spans="6:16" x14ac:dyDescent="0.3">
+      <c r="F23" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adding textbox input, still working
</commit_message>
<xml_diff>
--- a/unit_tests/test_cases.xlsx
+++ b/unit_tests/test_cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aa4f6975e0189fcb/Documents/Source/Cars/unit_tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="109" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{630AFC59-4944-4545-A9A6-9EE4B8B1867D}"/>
+  <xr:revisionPtr revIDLastSave="127" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{85D79C25-3AA7-4888-96C5-1C13836F6172}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="8880" activeTab="4" xr2:uid="{E1449062-40AE-488A-A0E8-5543147B756E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{E1449062-40AE-488A-A0E8-5543147B756E}"/>
   </bookViews>
   <sheets>
     <sheet name="TC-D5" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,8 @@
     <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
     <sheet name="Design" sheetId="5" r:id="rId4"/>
     <sheet name="Database-Design" sheetId="6" r:id="rId5"/>
-    <sheet name="CoordinateDirection" sheetId="4" r:id="rId6"/>
+    <sheet name="App-Design" sheetId="7" r:id="rId6"/>
+    <sheet name="CoordinateDirection" sheetId="4" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="82">
   <si>
     <t>Gallon per mile</t>
   </si>
@@ -266,6 +267,27 @@
   </si>
   <si>
     <t>Assign the car above with ending X and Y</t>
+  </si>
+  <si>
+    <t>Car game</t>
+  </si>
+  <si>
+    <t xml:space="preserve">database </t>
+  </si>
+  <si>
+    <t>car explorer</t>
+  </si>
+  <si>
+    <t>&lt;-----&gt;</t>
+  </si>
+  <si>
+    <t>app layer</t>
+  </si>
+  <si>
+    <t>database layer</t>
+  </si>
+  <si>
+    <t>CRUD</t>
   </si>
 </sst>
 </file>
@@ -297,7 +319,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -305,11 +327,91 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -318,6 +420,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1695,6 +1806,86 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EED5C1B-0A68-4559-9466-4CCE32F032D5}">
+  <dimension ref="F3:P9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="3" spans="6:16" x14ac:dyDescent="0.3">
+      <c r="F3" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G3" s="9"/>
+      <c r="H3" s="5"/>
+    </row>
+    <row r="4" spans="6:16" x14ac:dyDescent="0.3">
+      <c r="F4" s="10"/>
+      <c r="G4" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="H4" s="11"/>
+    </row>
+    <row r="5" spans="6:16" x14ac:dyDescent="0.3">
+      <c r="F5" s="10"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="11"/>
+    </row>
+    <row r="6" spans="6:16" x14ac:dyDescent="0.3">
+      <c r="F6" s="10"/>
+      <c r="G6" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="H6" s="11"/>
+      <c r="J6" t="s">
+        <v>78</v>
+      </c>
+      <c r="L6" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="M6" s="9"/>
+      <c r="N6" s="9"/>
+      <c r="O6" s="9"/>
+      <c r="P6" s="5"/>
+    </row>
+    <row r="7" spans="6:16" x14ac:dyDescent="0.3">
+      <c r="F7" s="10"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="L7" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="11"/>
+    </row>
+    <row r="8" spans="6:16" x14ac:dyDescent="0.3">
+      <c r="F8" s="10"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="11"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="11"/>
+    </row>
+    <row r="9" spans="6:16" x14ac:dyDescent="0.3">
+      <c r="F9" s="6"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="7"/>
+      <c r="L9" s="6"/>
+      <c r="M9" s="12"/>
+      <c r="N9" s="12"/>
+      <c r="O9" s="12"/>
+      <c r="P9" s="7"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1643BAB-DCF5-4FE9-88FC-DB471EA141B5}">
   <dimension ref="F10:L15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
Before refactoring for Car Game files
</commit_message>
<xml_diff>
--- a/unit_tests/test_cases.xlsx
+++ b/unit_tests/test_cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aa4f6975e0189fcb/Documents/Source/Cars/unit_tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="127" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{85D79C25-3AA7-4888-96C5-1C13836F6172}"/>
+  <xr:revisionPtr revIDLastSave="138" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3118CDEA-0219-4552-99E5-26F29764CC9E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{E1449062-40AE-488A-A0E8-5543147B756E}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="85">
   <si>
     <t>Gallon per mile</t>
   </si>
@@ -288,6 +288,15 @@
   </si>
   <si>
     <t>CRUD</t>
+  </si>
+  <si>
+    <t>main.py</t>
+  </si>
+  <si>
+    <t>List of Positions</t>
+  </si>
+  <si>
+    <t>CarGame(destinations)</t>
   </si>
 </sst>
 </file>
@@ -414,21 +423,21 @@
   <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1807,78 +1816,96 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EED5C1B-0A68-4559-9466-4CCE32F032D5}">
-  <dimension ref="F3:P9"/>
+  <dimension ref="B3:P9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="3" spans="6:16" x14ac:dyDescent="0.3">
-      <c r="F3" s="4" t="s">
+    <row r="3" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B3" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C3" s="6"/>
+      <c r="D3" s="3"/>
+      <c r="F3" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="G3" s="9"/>
-      <c r="H3" s="5"/>
-    </row>
-    <row r="4" spans="6:16" x14ac:dyDescent="0.3">
-      <c r="F4" s="10"/>
-      <c r="G4" s="8" t="s">
+      <c r="G3" s="6"/>
+      <c r="H3" s="3"/>
+    </row>
+    <row r="4" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B4" s="7"/>
+      <c r="C4" t="s">
+        <v>83</v>
+      </c>
+      <c r="D4" s="8"/>
+      <c r="F4" s="7"/>
+      <c r="G4" t="s">
         <v>79</v>
       </c>
-      <c r="H4" s="11"/>
-    </row>
-    <row r="5" spans="6:16" x14ac:dyDescent="0.3">
-      <c r="F5" s="10"/>
-      <c r="G5" s="8"/>
-      <c r="H5" s="11"/>
-    </row>
-    <row r="6" spans="6:16" x14ac:dyDescent="0.3">
-      <c r="F6" s="10"/>
-      <c r="G6" s="8" t="s">
+      <c r="H4" s="8"/>
+    </row>
+    <row r="5" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B5" s="7"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="8"/>
+      <c r="F5" s="7"/>
+      <c r="H5" s="8"/>
+    </row>
+    <row r="6" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B6" s="7"/>
+      <c r="C6" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="D6" s="8"/>
+      <c r="F6" s="7"/>
+      <c r="G6" t="s">
         <v>80</v>
       </c>
-      <c r="H6" s="11"/>
+      <c r="H6" s="8"/>
       <c r="J6" t="s">
         <v>78</v>
       </c>
-      <c r="L6" s="4" t="s">
+      <c r="L6" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="M6" s="9"/>
-      <c r="N6" s="9"/>
-      <c r="O6" s="9"/>
-      <c r="P6" s="5"/>
-    </row>
-    <row r="7" spans="6:16" x14ac:dyDescent="0.3">
-      <c r="F7" s="10"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="11" t="s">
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="3"/>
+    </row>
+    <row r="7" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B7" s="7"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="8"/>
+      <c r="F7" s="7"/>
+      <c r="H7" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="L7" s="10" t="s">
+      <c r="L7" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="M7" s="8"/>
-      <c r="N7" s="8"/>
-      <c r="O7" s="8"/>
-      <c r="P7" s="11"/>
-    </row>
-    <row r="8" spans="6:16" x14ac:dyDescent="0.3">
-      <c r="F8" s="10"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="11"/>
-      <c r="L8" s="10"/>
-      <c r="M8" s="8"/>
-      <c r="N8" s="8"/>
-      <c r="O8" s="8"/>
-      <c r="P8" s="11"/>
-    </row>
-    <row r="9" spans="6:16" x14ac:dyDescent="0.3">
-      <c r="F9" s="6"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="7"/>
-      <c r="L9" s="6"/>
-      <c r="M9" s="12"/>
-      <c r="N9" s="12"/>
-      <c r="O9" s="12"/>
-      <c r="P9" s="7"/>
+      <c r="P7" s="8"/>
+    </row>
+    <row r="8" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B8" s="7"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="8"/>
+      <c r="F8" s="7"/>
+      <c r="H8" s="8"/>
+      <c r="L8" s="7"/>
+      <c r="P8" s="8"/>
+    </row>
+    <row r="9" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B9" s="4"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="5"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="5"/>
+      <c r="L9" s="4"/>
+      <c r="M9" s="9"/>
+      <c r="N9" s="9"/>
+      <c r="O9" s="9"/>
+      <c r="P9" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1896,12 +1923,12 @@
   </cols>
   <sheetData>
     <row r="10" spans="6:12" x14ac:dyDescent="0.3">
-      <c r="I10" s="2" t="s">
+      <c r="I10" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="10"/>
+      <c r="L10" s="10"/>
     </row>
     <row r="11" spans="6:12" x14ac:dyDescent="0.3">
       <c r="I11" s="1" t="s">
@@ -1918,7 +1945,7 @@
       </c>
     </row>
     <row r="12" spans="6:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="11" t="s">
         <v>21</v>
       </c>
       <c r="G12" s="1" t="s">
@@ -1940,7 +1967,7 @@
       </c>
     </row>
     <row r="13" spans="6:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F13" s="3"/>
+      <c r="F13" s="11"/>
       <c r="G13" s="1" t="s">
         <v>34</v>
       </c>
@@ -1960,7 +1987,7 @@
       </c>
     </row>
     <row r="14" spans="6:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F14" s="3"/>
+      <c r="F14" s="11"/>
       <c r="G14" s="1" t="s">
         <v>35</v>
       </c>
@@ -1980,7 +2007,7 @@
       </c>
     </row>
     <row r="15" spans="6:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F15" s="3"/>
+      <c r="F15" s="11"/>
       <c r="G15" s="1" t="s">
         <v>36</v>
       </c>

</xml_diff>

<commit_message>
before reducing main files
</commit_message>
<xml_diff>
--- a/unit_tests/test_cases.xlsx
+++ b/unit_tests/test_cases.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aa4f6975e0189fcb/Documents/Source/Cars/unit_tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="138" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3118CDEA-0219-4552-99E5-26F29764CC9E}"/>
+  <xr:revisionPtr revIDLastSave="199" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0D95E89E-BE93-4DD0-B1E8-717C0954BE5E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{E1449062-40AE-488A-A0E8-5543147B756E}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="103">
   <si>
     <t>Gallon per mile</t>
   </si>
@@ -297,6 +297,60 @@
   </si>
   <si>
     <t>CarGame(destinations)</t>
+  </si>
+  <si>
+    <t>Game  (Run game)</t>
+  </si>
+  <si>
+    <t>AiSetting</t>
+  </si>
+  <si>
+    <t>Screen</t>
+  </si>
+  <si>
+    <t>Car explorer</t>
+  </si>
+  <si>
+    <t>Map</t>
+  </si>
+  <si>
+    <t>Status 1</t>
+  </si>
+  <si>
+    <t>Status 2</t>
+  </si>
+  <si>
+    <t>Status N</t>
+  </si>
+  <si>
+    <t>Seattle</t>
+  </si>
+  <si>
+    <t>Los Angeles</t>
+  </si>
+  <si>
+    <t>Atlanta</t>
+  </si>
+  <si>
+    <t>New York</t>
+  </si>
+  <si>
+    <t>(x,y)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">top, left </t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>draw_rectangle(position, w, h)</t>
+  </si>
+  <si>
+    <t>self.map.draw_rectange(self.position, w, h)</t>
+  </si>
+  <si>
+    <t>show(self)</t>
   </si>
 </sst>
 </file>
@@ -320,15 +374,27 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -416,11 +482,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -431,13 +512,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1816,96 +1900,293 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EED5C1B-0A68-4559-9466-4CCE32F032D5}">
-  <dimension ref="B3:P9"/>
+  <dimension ref="F3:T44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="3" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B3" s="2" t="s">
+    <row r="3" spans="6:20" x14ac:dyDescent="0.3">
+      <c r="F3" s="2" t="s">
         <v>82</v>
-      </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="3"/>
-      <c r="F3" s="2" t="s">
-        <v>75</v>
       </c>
       <c r="G3" s="6"/>
       <c r="H3" s="3"/>
-    </row>
-    <row r="4" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B4" s="7"/>
-      <c r="C4" t="s">
-        <v>83</v>
-      </c>
-      <c r="D4" s="8"/>
+      <c r="J3" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K3" s="6"/>
+      <c r="L3" s="3"/>
+    </row>
+    <row r="4" spans="6:20" x14ac:dyDescent="0.3">
       <c r="F4" s="7"/>
       <c r="G4" t="s">
+        <v>83</v>
+      </c>
+      <c r="H4" s="8"/>
+      <c r="J4" s="7"/>
+      <c r="K4" t="s">
         <v>79</v>
       </c>
-      <c r="H4" s="8"/>
-    </row>
-    <row r="5" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B5" s="7"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="8"/>
+      <c r="L4" s="8"/>
+    </row>
+    <row r="5" spans="6:20" x14ac:dyDescent="0.3">
       <c r="F5" s="7"/>
       <c r="H5" s="8"/>
-    </row>
-    <row r="6" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B6" s="7"/>
-      <c r="C6" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="D6" s="8"/>
+      <c r="J5" s="7"/>
+      <c r="L5" s="8"/>
+    </row>
+    <row r="6" spans="6:20" x14ac:dyDescent="0.3">
       <c r="F6" s="7"/>
       <c r="G6" t="s">
+        <v>84</v>
+      </c>
+      <c r="H6" s="8"/>
+      <c r="J6" s="7"/>
+      <c r="K6" t="s">
         <v>80</v>
       </c>
-      <c r="H6" s="8"/>
-      <c r="J6" t="s">
+      <c r="L6" s="8"/>
+      <c r="N6" t="s">
         <v>78</v>
       </c>
-      <c r="L6" s="2" t="s">
+      <c r="P6" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="M6" s="6"/>
-      <c r="N6" s="6"/>
-      <c r="O6" s="6"/>
-      <c r="P6" s="3"/>
-    </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B7" s="7"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="8"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="6"/>
+      <c r="S6" s="6"/>
+      <c r="T6" s="3"/>
+    </row>
+    <row r="7" spans="6:20" x14ac:dyDescent="0.3">
       <c r="F7" s="7"/>
-      <c r="H7" s="8" t="s">
+      <c r="H7" s="8"/>
+      <c r="J7" s="7"/>
+      <c r="L7" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="L7" s="7" t="s">
+      <c r="P7" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="P7" s="8"/>
-    </row>
-    <row r="8" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B8" s="7"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="8"/>
+      <c r="T7" s="8"/>
+    </row>
+    <row r="8" spans="6:20" x14ac:dyDescent="0.3">
       <c r="F8" s="7"/>
       <c r="H8" s="8"/>
-      <c r="L8" s="7"/>
-      <c r="P8" s="8"/>
-    </row>
-    <row r="9" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B9" s="4"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="5"/>
+      <c r="J8" s="7"/>
+      <c r="L8" s="8"/>
+      <c r="P8" s="7"/>
+      <c r="T8" s="8"/>
+    </row>
+    <row r="9" spans="6:20" x14ac:dyDescent="0.3">
       <c r="F9" s="4"/>
       <c r="G9" s="9"/>
       <c r="H9" s="5"/>
-      <c r="L9" s="4"/>
-      <c r="M9" s="9"/>
-      <c r="N9" s="9"/>
-      <c r="O9" s="9"/>
-      <c r="P9" s="5"/>
+      <c r="J9" s="4"/>
+      <c r="K9" s="9"/>
+      <c r="L9" s="5"/>
+      <c r="P9" s="4"/>
+      <c r="Q9" s="9"/>
+      <c r="R9" s="9"/>
+      <c r="S9" s="9"/>
+      <c r="T9" s="5"/>
+    </row>
+    <row r="13" spans="6:20" x14ac:dyDescent="0.3">
+      <c r="G13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="15" spans="6:20" x14ac:dyDescent="0.3">
+      <c r="G15" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" spans="7:17" x14ac:dyDescent="0.3">
+      <c r="G17" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="19" spans="7:17" x14ac:dyDescent="0.3">
+      <c r="G19" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="H19" s="6"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="6"/>
+      <c r="K19" s="6"/>
+      <c r="L19" s="6"/>
+      <c r="M19" s="6"/>
+      <c r="N19" s="6"/>
+      <c r="O19" s="3"/>
+    </row>
+    <row r="20" spans="7:17" x14ac:dyDescent="0.3">
+      <c r="G20" s="7"/>
+      <c r="H20" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="I20" s="11"/>
+      <c r="J20" s="11"/>
+      <c r="K20" s="11"/>
+      <c r="L20" s="11"/>
+      <c r="O20" s="8"/>
+    </row>
+    <row r="21" spans="7:17" x14ac:dyDescent="0.3">
+      <c r="G21" s="7"/>
+      <c r="H21" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="I21" s="11"/>
+      <c r="J21" s="11"/>
+      <c r="K21" s="11"/>
+      <c r="L21" s="11"/>
+      <c r="O21" s="8"/>
+    </row>
+    <row r="22" spans="7:17" x14ac:dyDescent="0.3">
+      <c r="G22" s="7"/>
+      <c r="H22" s="11"/>
+      <c r="I22" s="11"/>
+      <c r="J22" s="11"/>
+      <c r="K22" s="12"/>
+      <c r="L22" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="O22" s="8"/>
+    </row>
+    <row r="23" spans="7:17" x14ac:dyDescent="0.3">
+      <c r="G23" s="7"/>
+      <c r="H23" s="11"/>
+      <c r="I23" s="11"/>
+      <c r="J23" s="11"/>
+      <c r="K23" s="11"/>
+      <c r="L23" s="11"/>
+      <c r="O23" s="8"/>
+    </row>
+    <row r="24" spans="7:17" x14ac:dyDescent="0.3">
+      <c r="G24" s="7"/>
+      <c r="H24" s="11"/>
+      <c r="I24" s="11"/>
+      <c r="J24" s="11"/>
+      <c r="K24" s="11"/>
+      <c r="L24" s="11"/>
+      <c r="N24" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="O24" s="8"/>
+      <c r="Q24" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="25" spans="7:17" x14ac:dyDescent="0.3">
+      <c r="G25" s="7"/>
+      <c r="H25" s="11"/>
+      <c r="I25" s="11"/>
+      <c r="J25" s="12"/>
+      <c r="K25" s="11"/>
+      <c r="L25" s="11"/>
+      <c r="N25" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="O25" s="8"/>
+    </row>
+    <row r="26" spans="7:17" x14ac:dyDescent="0.3">
+      <c r="G26" s="7"/>
+      <c r="H26" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="I26" s="11"/>
+      <c r="J26" s="11"/>
+      <c r="K26" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="L26" s="11"/>
+      <c r="N26" s="10"/>
+      <c r="O26" s="8"/>
+    </row>
+    <row r="27" spans="7:17" x14ac:dyDescent="0.3">
+      <c r="G27" s="7"/>
+      <c r="H27" s="11"/>
+      <c r="I27" s="11"/>
+      <c r="J27" s="11"/>
+      <c r="K27" s="11"/>
+      <c r="L27" s="11"/>
+      <c r="N27" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="O27" s="8"/>
+    </row>
+    <row r="28" spans="7:17" x14ac:dyDescent="0.3">
+      <c r="G28" s="7"/>
+      <c r="H28" s="11"/>
+      <c r="I28" s="11"/>
+      <c r="J28" s="11"/>
+      <c r="K28" s="11"/>
+      <c r="L28" s="11"/>
+      <c r="O28" s="8"/>
+    </row>
+    <row r="29" spans="7:17" x14ac:dyDescent="0.3">
+      <c r="G29" s="4"/>
+      <c r="H29" s="9"/>
+      <c r="I29" s="9"/>
+      <c r="J29" s="9"/>
+      <c r="K29" s="9"/>
+      <c r="L29" s="9"/>
+      <c r="M29" s="9"/>
+      <c r="N29" s="9"/>
+      <c r="O29" s="5"/>
+    </row>
+    <row r="32" spans="7:17" x14ac:dyDescent="0.3">
+      <c r="H32" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="33" spans="8:11" x14ac:dyDescent="0.3">
+      <c r="I33" s="12"/>
+      <c r="J33" s="12"/>
+      <c r="K33" s="12"/>
+    </row>
+    <row r="34" spans="8:11" x14ac:dyDescent="0.3">
+      <c r="I34" s="12"/>
+      <c r="J34" s="12"/>
+      <c r="K34" s="12"/>
+    </row>
+    <row r="35" spans="8:11" x14ac:dyDescent="0.3">
+      <c r="I35" s="12"/>
+      <c r="J35" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="K35" s="12"/>
+    </row>
+    <row r="36" spans="8:11" x14ac:dyDescent="0.3">
+      <c r="I36" s="12"/>
+      <c r="J36" s="12"/>
+      <c r="K36" s="12"/>
+    </row>
+    <row r="37" spans="8:11" x14ac:dyDescent="0.3">
+      <c r="I37" s="12"/>
+      <c r="J37" s="12"/>
+      <c r="K37" s="12"/>
+    </row>
+    <row r="39" spans="8:11" x14ac:dyDescent="0.3">
+      <c r="H39" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="40" spans="8:11" x14ac:dyDescent="0.3">
+      <c r="I40" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="42" spans="8:11" x14ac:dyDescent="0.3">
+      <c r="H42" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="43" spans="8:11" x14ac:dyDescent="0.3">
+      <c r="I43" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="44" spans="8:11" x14ac:dyDescent="0.3">
+      <c r="J44" t="s">
+        <v>101</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1923,12 +2204,12 @@
   </cols>
   <sheetData>
     <row r="10" spans="6:12" x14ac:dyDescent="0.3">
-      <c r="I10" s="10" t="s">
+      <c r="I10" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="J10" s="10"/>
-      <c r="K10" s="10"/>
-      <c r="L10" s="10"/>
+      <c r="J10" s="14"/>
+      <c r="K10" s="14"/>
+      <c r="L10" s="14"/>
     </row>
     <row r="11" spans="6:12" x14ac:dyDescent="0.3">
       <c r="I11" s="1" t="s">
@@ -1945,7 +2226,7 @@
       </c>
     </row>
     <row r="12" spans="6:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F12" s="11" t="s">
+      <c r="F12" s="15" t="s">
         <v>21</v>
       </c>
       <c r="G12" s="1" t="s">
@@ -1967,7 +2248,7 @@
       </c>
     </row>
     <row r="13" spans="6:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F13" s="11"/>
+      <c r="F13" s="15"/>
       <c r="G13" s="1" t="s">
         <v>34</v>
       </c>
@@ -1987,7 +2268,7 @@
       </c>
     </row>
     <row r="14" spans="6:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F14" s="11"/>
+      <c r="F14" s="15"/>
       <c r="G14" s="1" t="s">
         <v>35</v>
       </c>
@@ -2007,7 +2288,7 @@
       </c>
     </row>
     <row r="15" spans="6:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F15" s="11"/>
+      <c r="F15" s="15"/>
       <c r="G15" s="1" t="s">
         <v>36</v>
       </c>

</xml_diff>

<commit_message>
added atlanta position and removed unnecessary for loop when drawing city
</commit_message>
<xml_diff>
--- a/unit_tests/test_cases.xlsx
+++ b/unit_tests/test_cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aa4f6975e0189fcb/Documents/Source/Cars/unit_tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="199" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0D95E89E-BE93-4DD0-B1E8-717C0954BE5E}"/>
+  <xr:revisionPtr revIDLastSave="208" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{587A9A0A-7D50-49AE-AB27-CAD3CF930BB9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{E1449062-40AE-488A-A0E8-5543147B756E}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="109">
   <si>
     <t>Gallon per mile</t>
   </si>
@@ -351,6 +351,24 @@
   </si>
   <si>
     <t>show(self)</t>
+  </si>
+  <si>
+    <t>Shape</t>
+  </si>
+  <si>
+    <t>screen</t>
+  </si>
+  <si>
+    <t>pygame</t>
+  </si>
+  <si>
+    <t>draw_rectangle</t>
+  </si>
+  <si>
+    <t>draw_text_on_rectangle</t>
+  </si>
+  <si>
+    <t>show</t>
   </si>
 </sst>
 </file>
@@ -1900,7 +1918,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EED5C1B-0A68-4559-9466-4CCE32F032D5}">
-  <dimension ref="F3:T44"/>
+  <dimension ref="D3:T45"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="3" spans="6:20" x14ac:dyDescent="0.3">
@@ -2136,56 +2154,78 @@
         <v>98</v>
       </c>
     </row>
-    <row r="33" spans="8:11" x14ac:dyDescent="0.3">
+    <row r="33" spans="4:11" x14ac:dyDescent="0.3">
       <c r="I33" s="12"/>
       <c r="J33" s="12"/>
       <c r="K33" s="12"/>
     </row>
-    <row r="34" spans="8:11" x14ac:dyDescent="0.3">
+    <row r="34" spans="4:11" x14ac:dyDescent="0.3">
       <c r="I34" s="12"/>
       <c r="J34" s="12"/>
       <c r="K34" s="12"/>
     </row>
-    <row r="35" spans="8:11" x14ac:dyDescent="0.3">
+    <row r="35" spans="4:11" x14ac:dyDescent="0.3">
       <c r="I35" s="12"/>
       <c r="J35" s="12" t="s">
         <v>97</v>
       </c>
       <c r="K35" s="12"/>
     </row>
-    <row r="36" spans="8:11" x14ac:dyDescent="0.3">
+    <row r="36" spans="4:11" x14ac:dyDescent="0.3">
       <c r="I36" s="12"/>
       <c r="J36" s="12"/>
       <c r="K36" s="12"/>
     </row>
-    <row r="37" spans="8:11" x14ac:dyDescent="0.3">
+    <row r="37" spans="4:11" x14ac:dyDescent="0.3">
       <c r="I37" s="12"/>
       <c r="J37" s="12"/>
       <c r="K37" s="12"/>
     </row>
-    <row r="39" spans="8:11" x14ac:dyDescent="0.3">
+    <row r="39" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="D39" t="s">
+        <v>103</v>
+      </c>
       <c r="H39" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="40" spans="8:11" x14ac:dyDescent="0.3">
+    <row r="40" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="E40" t="s">
+        <v>104</v>
+      </c>
       <c r="I40" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="42" spans="8:11" x14ac:dyDescent="0.3">
+    <row r="41" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="E41" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="42" spans="4:11" x14ac:dyDescent="0.3">
       <c r="H42" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="43" spans="8:11" x14ac:dyDescent="0.3">
+    <row r="43" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="E43" t="s">
+        <v>106</v>
+      </c>
       <c r="I43" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="44" spans="8:11" x14ac:dyDescent="0.3">
+    <row r="44" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="E44" t="s">
+        <v>107</v>
+      </c>
       <c r="J44" t="s">
         <v>101</v>
+      </c>
+    </row>
+    <row r="45" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="E45" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adding shape and draw rectangle and text
</commit_message>
<xml_diff>
--- a/unit_tests/test_cases.xlsx
+++ b/unit_tests/test_cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aa4f6975e0189fcb/Documents/Source/Cars/unit_tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="208" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{587A9A0A-7D50-49AE-AB27-CAD3CF930BB9}"/>
+  <xr:revisionPtr revIDLastSave="216" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{586698B7-D50B-41B9-8FC1-E2386909593B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{E1449062-40AE-488A-A0E8-5543147B756E}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="114">
   <si>
     <t>Gallon per mile</t>
   </si>
@@ -369,6 +369,21 @@
   </si>
   <si>
     <t>show</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>position</t>
+  </si>
+  <si>
+    <t>Car</t>
+  </si>
+  <si>
+    <t>Person</t>
   </si>
 </sst>
 </file>
@@ -1918,7 +1933,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EED5C1B-0A68-4559-9466-4CCE32F032D5}">
-  <dimension ref="D3:T45"/>
+  <dimension ref="D3:T49"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="3" spans="6:20" x14ac:dyDescent="0.3">
@@ -2203,13 +2218,16 @@
       </c>
     </row>
     <row r="42" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="E42" t="s">
+        <v>109</v>
+      </c>
       <c r="H42" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="43" spans="4:11" x14ac:dyDescent="0.3">
       <c r="E43" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="I43" t="s">
         <v>102</v>
@@ -2217,15 +2235,33 @@
     </row>
     <row r="44" spans="4:11" x14ac:dyDescent="0.3">
       <c r="E44" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="J44" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="45" spans="4:11" x14ac:dyDescent="0.3">
-      <c r="E45" t="s">
+    <row r="46" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="H46" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="47" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="E47" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="48" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="E48" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="49" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E49" t="s">
         <v>108</v>
+      </c>
+      <c r="H49" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
created draw point function, simplified city call clutter in other classes and methods, and create triangle and pentagon in pygame window
</commit_message>
<xml_diff>
--- a/unit_tests/test_cases.xlsx
+++ b/unit_tests/test_cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aa4f6975e0189fcb/Documents/Source/Cars/unit_tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="216" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{586698B7-D50B-41B9-8FC1-E2386909593B}"/>
+  <xr:revisionPtr revIDLastSave="248" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40179080-DB28-493D-8B3C-83E69A04AC9D}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{E1449062-40AE-488A-A0E8-5543147B756E}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="129">
   <si>
     <t>Gallon per mile</t>
   </si>
@@ -194,12 +194,6 @@
     <t>game</t>
   </si>
   <si>
-    <t>component</t>
-  </si>
-  <si>
-    <t>factory</t>
-  </si>
-  <si>
     <t>Table</t>
   </si>
   <si>
@@ -384,6 +378,57 @@
   </si>
   <si>
     <t>Person</t>
+  </si>
+  <si>
+    <t>Instance variables</t>
+  </si>
+  <si>
+    <t>game.Cities</t>
+  </si>
+  <si>
+    <t>CityID</t>
+  </si>
+  <si>
+    <t>All the fields in the City class</t>
+  </si>
+  <si>
+    <t>Car Explorer, Data Access Layer (DAL), Data Access Object (DAO)</t>
+  </si>
+  <si>
+    <t>get_cities</t>
+  </si>
+  <si>
+    <t>get all cities</t>
+  </si>
+  <si>
+    <t xml:space="preserve">for each city </t>
+  </si>
+  <si>
+    <t>build a city object</t>
+  </si>
+  <si>
+    <t>return all cities</t>
+  </si>
+  <si>
+    <t>CityRepo, Data Access Layer (DAL), Data Access Object (DAO)</t>
+  </si>
+  <si>
+    <t>CityRepo</t>
+  </si>
+  <si>
+    <t>Cities</t>
+  </si>
+  <si>
+    <t>dto</t>
+  </si>
+  <si>
+    <t>Builder</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>CityDto</t>
   </si>
 </sst>
 </file>
@@ -1768,162 +1813,204 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C68B0F5-EBBE-43FB-B76D-76A1F84FE911}">
-  <dimension ref="F1:P23"/>
+  <dimension ref="C1:P32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="4" max="4" width="11.5546875" customWidth="1"/>
     <col min="6" max="6" width="13.44140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="6:15" x14ac:dyDescent="0.3">
-      <c r="F1" t="s">
+    <row r="1" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="C1" t="s">
         <v>46</v>
       </c>
-      <c r="G1" t="s">
+      <c r="D1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="6:15" x14ac:dyDescent="0.3">
-      <c r="F3" t="s">
+    <row r="3" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="D3" t="s">
         <v>48</v>
       </c>
-      <c r="G3" t="s">
+      <c r="E3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="E5" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="7" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="F7" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="4" spans="6:15" x14ac:dyDescent="0.3">
-      <c r="G4" t="s">
+      <c r="G7" t="s">
+        <v>53</v>
+      </c>
+      <c r="H7" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="5" spans="6:15" x14ac:dyDescent="0.3">
-      <c r="G5" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="8" spans="6:15" x14ac:dyDescent="0.3">
-      <c r="F8" t="s">
+      <c r="I7" t="s">
+        <v>55</v>
+      </c>
+      <c r="J7" t="s">
         <v>52</v>
       </c>
+      <c r="K7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" spans="3:15" x14ac:dyDescent="0.3">
       <c r="G8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H8" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="I8" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="J8" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="K8" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" spans="6:15" x14ac:dyDescent="0.3">
-      <c r="G9" t="s">
-        <v>56</v>
-      </c>
-      <c r="H9" t="s">
         <v>59</v>
       </c>
-      <c r="I9" t="s">
-        <v>53</v>
-      </c>
-      <c r="J9" t="s">
+      <c r="L8" t="s">
         <v>60</v>
       </c>
-      <c r="K9" t="s">
+      <c r="M8" t="s">
         <v>61</v>
       </c>
-      <c r="L9" t="s">
+      <c r="N8" t="s">
         <v>62</v>
       </c>
-      <c r="M9" t="s">
+      <c r="O8" t="s">
         <v>63</v>
       </c>
-      <c r="N9" t="s">
+    </row>
+    <row r="11" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="F11" t="s">
         <v>64</v>
       </c>
-      <c r="O9" t="s">
+    </row>
+    <row r="12" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="F12" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="6:15" x14ac:dyDescent="0.3">
-      <c r="F12" t="s">
+    <row r="13" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="G13" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="13" spans="6:15" x14ac:dyDescent="0.3">
-      <c r="F13" t="s">
+    <row r="14" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="F14" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="14" spans="6:15" x14ac:dyDescent="0.3">
-      <c r="G14" t="s">
+    <row r="15" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="G15" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="6:15" x14ac:dyDescent="0.3">
-      <c r="F15" t="s">
+    <row r="16" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="F16" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18" spans="5:16" x14ac:dyDescent="0.3">
+      <c r="F18" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="16" spans="6:15" x14ac:dyDescent="0.3">
-      <c r="G16" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="17" spans="6:16" x14ac:dyDescent="0.3">
-      <c r="F17" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="19" spans="6:16" x14ac:dyDescent="0.3">
+    <row r="19" spans="5:16" x14ac:dyDescent="0.3">
       <c r="F19" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="20" spans="6:16" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="20" spans="5:16" x14ac:dyDescent="0.3">
       <c r="F20" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="21" spans="6:16" x14ac:dyDescent="0.3">
-      <c r="F21" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="22" spans="6:16" x14ac:dyDescent="0.3">
-      <c r="G22" t="s">
+    <row r="21" spans="5:16" x14ac:dyDescent="0.3">
+      <c r="G21" t="s">
+        <v>70</v>
+      </c>
+      <c r="I21" t="s">
+        <v>57</v>
+      </c>
+      <c r="K21" t="s">
+        <v>58</v>
+      </c>
+      <c r="L21" t="s">
+        <v>59</v>
+      </c>
+      <c r="M21" t="s">
+        <v>60</v>
+      </c>
+      <c r="N21" t="s">
+        <v>61</v>
+      </c>
+      <c r="O21" t="s">
+        <v>62</v>
+      </c>
+      <c r="P21" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="22" spans="5:16" x14ac:dyDescent="0.3">
+      <c r="F22" t="s">
         <v>72</v>
       </c>
-      <c r="I22" t="s">
-        <v>59</v>
-      </c>
-      <c r="K22" t="s">
-        <v>60</v>
-      </c>
-      <c r="L22" t="s">
-        <v>61</v>
-      </c>
-      <c r="M22" t="s">
-        <v>62</v>
-      </c>
-      <c r="N22" t="s">
-        <v>63</v>
-      </c>
-      <c r="O22" t="s">
-        <v>64</v>
-      </c>
-      <c r="P22" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="23" spans="6:16" x14ac:dyDescent="0.3">
-      <c r="F23" t="s">
-        <v>74</v>
+    </row>
+    <row r="24" spans="5:16" x14ac:dyDescent="0.3">
+      <c r="E24" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="25" spans="5:16" x14ac:dyDescent="0.3">
+      <c r="F25" t="s">
+        <v>50</v>
+      </c>
+      <c r="G25" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="26" spans="5:16" x14ac:dyDescent="0.3">
+      <c r="H26" t="s">
+        <v>114</v>
+      </c>
+      <c r="I26" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="28" spans="5:16" x14ac:dyDescent="0.3">
+      <c r="F28" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="29" spans="5:16" x14ac:dyDescent="0.3">
+      <c r="G29" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="30" spans="5:16" x14ac:dyDescent="0.3">
+      <c r="G30" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="31" spans="5:16" x14ac:dyDescent="0.3">
+      <c r="H31" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="32" spans="5:16" x14ac:dyDescent="0.3">
+      <c r="H32" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -1933,17 +2020,17 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EED5C1B-0A68-4559-9466-4CCE32F032D5}">
-  <dimension ref="D3:T49"/>
+  <dimension ref="D3:T55"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="3" spans="6:20" x14ac:dyDescent="0.3">
       <c r="F3" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G3" s="6"/>
       <c r="H3" s="3"/>
       <c r="J3" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K3" s="6"/>
       <c r="L3" s="3"/>
@@ -1951,12 +2038,12 @@
     <row r="4" spans="6:20" x14ac:dyDescent="0.3">
       <c r="F4" s="7"/>
       <c r="G4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="H4" s="8"/>
       <c r="J4" s="7"/>
       <c r="K4" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L4" s="8"/>
     </row>
@@ -1964,24 +2051,26 @@
       <c r="F5" s="7"/>
       <c r="H5" s="8"/>
       <c r="J5" s="7"/>
-      <c r="L5" s="8"/>
+      <c r="L5" s="8" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="6" spans="6:20" x14ac:dyDescent="0.3">
       <c r="F6" s="7"/>
       <c r="G6" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="H6" s="8"/>
       <c r="J6" s="7"/>
       <c r="K6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="L6" s="8"/>
       <c r="N6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
@@ -1993,10 +2082,10 @@
       <c r="H7" s="8"/>
       <c r="J7" s="7"/>
       <c r="L7" s="8" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="P7" s="7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="T7" s="8"/>
     </row>
@@ -2004,8 +2093,12 @@
       <c r="F8" s="7"/>
       <c r="H8" s="8"/>
       <c r="J8" s="7"/>
-      <c r="L8" s="8"/>
-      <c r="P8" s="7"/>
+      <c r="L8" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="P8" s="7" t="s">
+        <v>124</v>
+      </c>
       <c r="T8" s="8"/>
     </row>
     <row r="9" spans="6:20" x14ac:dyDescent="0.3">
@@ -2023,7 +2116,7 @@
     </row>
     <row r="13" spans="6:20" x14ac:dyDescent="0.3">
       <c r="G13" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="15" spans="6:20" x14ac:dyDescent="0.3">
@@ -2033,12 +2126,12 @@
     </row>
     <row r="17" spans="7:17" x14ac:dyDescent="0.3">
       <c r="G17" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="19" spans="7:17" x14ac:dyDescent="0.3">
       <c r="G19" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="H19" s="6"/>
       <c r="I19" s="6"/>
@@ -2052,7 +2145,7 @@
     <row r="20" spans="7:17" x14ac:dyDescent="0.3">
       <c r="G20" s="7"/>
       <c r="H20" s="11" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="I20" s="11"/>
       <c r="J20" s="11"/>
@@ -2063,7 +2156,7 @@
     <row r="21" spans="7:17" x14ac:dyDescent="0.3">
       <c r="G21" s="7"/>
       <c r="H21" s="13" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="I21" s="11"/>
       <c r="J21" s="11"/>
@@ -2078,7 +2171,7 @@
       <c r="J22" s="11"/>
       <c r="K22" s="12"/>
       <c r="L22" s="13" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="O22" s="8"/>
     </row>
@@ -2099,11 +2192,11 @@
       <c r="K24" s="11"/>
       <c r="L24" s="11"/>
       <c r="N24" s="10" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="O24" s="8"/>
       <c r="Q24" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="25" spans="7:17" x14ac:dyDescent="0.3">
@@ -2114,19 +2207,19 @@
       <c r="K25" s="11"/>
       <c r="L25" s="11"/>
       <c r="N25" s="10" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="O25" s="8"/>
     </row>
     <row r="26" spans="7:17" x14ac:dyDescent="0.3">
       <c r="G26" s="7"/>
       <c r="H26" s="13" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="I26" s="11"/>
       <c r="J26" s="11"/>
       <c r="K26" s="13" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="L26" s="11"/>
       <c r="N26" s="10"/>
@@ -2140,7 +2233,7 @@
       <c r="K27" s="11"/>
       <c r="L27" s="11"/>
       <c r="N27" s="10" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="O27" s="8"/>
     </row>
@@ -2166,7 +2259,7 @@
     </row>
     <row r="32" spans="7:17" x14ac:dyDescent="0.3">
       <c r="H32" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="33" spans="4:11" x14ac:dyDescent="0.3">
@@ -2182,7 +2275,7 @@
     <row r="35" spans="4:11" x14ac:dyDescent="0.3">
       <c r="I35" s="12"/>
       <c r="J35" s="12" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="K35" s="12"/>
     </row>
@@ -2198,70 +2291,91 @@
     </row>
     <row r="39" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D39" t="s">
-        <v>103</v>
+        <v>101</v>
+      </c>
+      <c r="E39" t="s">
+        <v>112</v>
       </c>
       <c r="H39" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="40" spans="4:11" x14ac:dyDescent="0.3">
       <c r="E40" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="I40" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="41" spans="4:11" x14ac:dyDescent="0.3">
       <c r="E41" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="42" spans="4:11" x14ac:dyDescent="0.3">
       <c r="E42" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="H42" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="43" spans="4:11" x14ac:dyDescent="0.3">
       <c r="E43" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="I43" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="44" spans="4:11" x14ac:dyDescent="0.3">
       <c r="E44" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="J44" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="46" spans="4:11" x14ac:dyDescent="0.3">
       <c r="H46" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="47" spans="4:11" x14ac:dyDescent="0.3">
       <c r="E47" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="48" spans="4:11" x14ac:dyDescent="0.3">
       <c r="E48" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="49" spans="5:8" x14ac:dyDescent="0.3">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="49" spans="4:8" x14ac:dyDescent="0.3">
       <c r="E49" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="H49" t="s">
-        <v>113</v>
+        <v>111</v>
+      </c>
+    </row>
+    <row r="53" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D53" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="54" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="E54" t="s">
+        <v>127</v>
+      </c>
+      <c r="G54" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="55" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="H55" t="s">
+        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
before create a base repo class
</commit_message>
<xml_diff>
--- a/unit_tests/test_cases.xlsx
+++ b/unit_tests/test_cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aa4f6975e0189fcb/Documents/Source/Cars/unit_tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="248" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40179080-DB28-493D-8B3C-83E69A04AC9D}"/>
+  <xr:revisionPtr revIDLastSave="305" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD77B93D-2575-4C7F-96E3-4A46EB12EB3B}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{E1449062-40AE-488A-A0E8-5543147B756E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{E1449062-40AE-488A-A0E8-5543147B756E}"/>
   </bookViews>
   <sheets>
     <sheet name="TC-D5" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,8 @@
     <sheet name="Design" sheetId="5" r:id="rId4"/>
     <sheet name="Database-Design" sheetId="6" r:id="rId5"/>
     <sheet name="App-Design" sheetId="7" r:id="rId6"/>
-    <sheet name="CoordinateDirection" sheetId="4" r:id="rId7"/>
+    <sheet name="Map" sheetId="8" r:id="rId7"/>
+    <sheet name="CoordinateDirection" sheetId="4" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -579,7 +580,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -599,6 +600,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2384,6 +2388,362 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B4D1224-06E7-451A-AAFD-053F2614A910}">
+  <dimension ref="A1:CW3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="144" width="2.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:101" x14ac:dyDescent="0.3">
+      <c r="A1">
+        <v>1</v>
+      </c>
+      <c r="B1">
+        <v>2</v>
+      </c>
+      <c r="C1">
+        <v>3</v>
+      </c>
+      <c r="D1">
+        <v>4</v>
+      </c>
+      <c r="E1">
+        <v>5</v>
+      </c>
+      <c r="F1">
+        <v>6</v>
+      </c>
+      <c r="G1">
+        <v>7</v>
+      </c>
+      <c r="H1">
+        <v>8</v>
+      </c>
+      <c r="I1">
+        <v>9</v>
+      </c>
+      <c r="J1">
+        <v>10</v>
+      </c>
+      <c r="K1">
+        <v>1</v>
+      </c>
+      <c r="L1">
+        <v>2</v>
+      </c>
+      <c r="M1">
+        <v>3</v>
+      </c>
+      <c r="N1">
+        <v>4</v>
+      </c>
+      <c r="O1">
+        <v>5</v>
+      </c>
+      <c r="P1">
+        <v>6</v>
+      </c>
+      <c r="Q1">
+        <v>7</v>
+      </c>
+      <c r="R1">
+        <v>8</v>
+      </c>
+      <c r="S1">
+        <v>9</v>
+      </c>
+      <c r="T1">
+        <v>10</v>
+      </c>
+      <c r="U1">
+        <v>1</v>
+      </c>
+      <c r="V1">
+        <v>2</v>
+      </c>
+      <c r="W1">
+        <v>3</v>
+      </c>
+      <c r="X1">
+        <v>4</v>
+      </c>
+      <c r="Y1">
+        <v>5</v>
+      </c>
+      <c r="Z1">
+        <v>6</v>
+      </c>
+      <c r="AA1">
+        <v>7</v>
+      </c>
+      <c r="AB1">
+        <v>8</v>
+      </c>
+      <c r="AC1">
+        <v>9</v>
+      </c>
+      <c r="AD1">
+        <v>10</v>
+      </c>
+      <c r="AE1">
+        <v>1</v>
+      </c>
+      <c r="AF1">
+        <v>2</v>
+      </c>
+      <c r="AG1">
+        <v>3</v>
+      </c>
+      <c r="AH1">
+        <v>4</v>
+      </c>
+      <c r="AI1">
+        <v>5</v>
+      </c>
+      <c r="AJ1">
+        <v>6</v>
+      </c>
+      <c r="AK1">
+        <v>7</v>
+      </c>
+      <c r="AL1">
+        <v>8</v>
+      </c>
+      <c r="AM1">
+        <v>9</v>
+      </c>
+      <c r="AN1">
+        <v>10</v>
+      </c>
+      <c r="AO1">
+        <v>1</v>
+      </c>
+      <c r="AP1">
+        <v>2</v>
+      </c>
+      <c r="AQ1">
+        <v>3</v>
+      </c>
+      <c r="AR1">
+        <v>4</v>
+      </c>
+      <c r="AS1">
+        <v>5</v>
+      </c>
+      <c r="AT1">
+        <v>6</v>
+      </c>
+      <c r="AU1">
+        <v>7</v>
+      </c>
+      <c r="AV1">
+        <v>8</v>
+      </c>
+      <c r="AW1">
+        <v>9</v>
+      </c>
+      <c r="AX1">
+        <v>10</v>
+      </c>
+      <c r="AY1">
+        <v>1</v>
+      </c>
+      <c r="AZ1">
+        <v>2</v>
+      </c>
+      <c r="BA1">
+        <v>3</v>
+      </c>
+      <c r="BB1">
+        <v>4</v>
+      </c>
+      <c r="BC1">
+        <v>5</v>
+      </c>
+      <c r="BD1">
+        <v>6</v>
+      </c>
+      <c r="BE1">
+        <v>7</v>
+      </c>
+      <c r="BF1">
+        <v>8</v>
+      </c>
+      <c r="BG1">
+        <v>9</v>
+      </c>
+      <c r="BH1">
+        <v>10</v>
+      </c>
+      <c r="BI1">
+        <v>1</v>
+      </c>
+      <c r="BJ1">
+        <v>2</v>
+      </c>
+      <c r="BK1">
+        <v>3</v>
+      </c>
+      <c r="BL1">
+        <v>4</v>
+      </c>
+      <c r="BM1">
+        <v>5</v>
+      </c>
+      <c r="BN1">
+        <v>6</v>
+      </c>
+      <c r="BO1">
+        <v>7</v>
+      </c>
+      <c r="BP1">
+        <v>8</v>
+      </c>
+      <c r="BQ1">
+        <v>9</v>
+      </c>
+      <c r="BR1">
+        <v>10</v>
+      </c>
+      <c r="BS1">
+        <v>1</v>
+      </c>
+      <c r="BT1">
+        <v>2</v>
+      </c>
+      <c r="BU1">
+        <v>3</v>
+      </c>
+      <c r="BV1">
+        <v>4</v>
+      </c>
+      <c r="BW1">
+        <v>5</v>
+      </c>
+      <c r="BX1">
+        <v>6</v>
+      </c>
+      <c r="BY1">
+        <v>7</v>
+      </c>
+      <c r="BZ1">
+        <v>8</v>
+      </c>
+      <c r="CA1">
+        <v>9</v>
+      </c>
+      <c r="CB1">
+        <v>10</v>
+      </c>
+      <c r="CC1">
+        <v>1</v>
+      </c>
+      <c r="CD1">
+        <v>2</v>
+      </c>
+      <c r="CE1">
+        <v>3</v>
+      </c>
+      <c r="CF1">
+        <v>4</v>
+      </c>
+      <c r="CG1">
+        <v>5</v>
+      </c>
+      <c r="CH1">
+        <v>6</v>
+      </c>
+      <c r="CI1">
+        <v>7</v>
+      </c>
+      <c r="CJ1">
+        <v>8</v>
+      </c>
+      <c r="CK1">
+        <v>9</v>
+      </c>
+      <c r="CL1">
+        <v>10</v>
+      </c>
+      <c r="CM1">
+        <v>1</v>
+      </c>
+      <c r="CN1">
+        <v>2</v>
+      </c>
+      <c r="CO1">
+        <v>3</v>
+      </c>
+      <c r="CP1">
+        <v>4</v>
+      </c>
+      <c r="CQ1">
+        <v>5</v>
+      </c>
+      <c r="CR1">
+        <v>6</v>
+      </c>
+      <c r="CS1">
+        <v>7</v>
+      </c>
+      <c r="CT1">
+        <v>8</v>
+      </c>
+      <c r="CU1">
+        <v>9</v>
+      </c>
+      <c r="CV1">
+        <v>10</v>
+      </c>
+      <c r="CW1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:101" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="U2">
+        <v>2</v>
+      </c>
+      <c r="AE2">
+        <v>3</v>
+      </c>
+      <c r="AO2">
+        <v>4</v>
+      </c>
+      <c r="AY2">
+        <v>5</v>
+      </c>
+      <c r="BI2">
+        <v>6</v>
+      </c>
+      <c r="BS2">
+        <v>7</v>
+      </c>
+      <c r="CC2">
+        <v>8</v>
+      </c>
+      <c r="CM2">
+        <v>9</v>
+      </c>
+      <c r="CW2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:101" x14ac:dyDescent="0.3">
+      <c r="K3" s="16"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1643BAB-DCF5-4FE9-88FC-DB471EA141B5}">
   <dimension ref="F10:L15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
added coding for position and travel distance to new position along with unit test
</commit_message>
<xml_diff>
--- a/unit_tests/test_cases.xlsx
+++ b/unit_tests/test_cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aa4f6975e0189fcb/Documents/Source/Cars/unit_tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="305" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD77B93D-2575-4C7F-96E3-4A46EB12EB3B}"/>
+  <xr:revisionPtr revIDLastSave="357" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{931E9543-C5CA-4AE8-BEB0-5CCB31AE1403}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{E1449062-40AE-488A-A0E8-5543147B756E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="5" xr2:uid="{E1449062-40AE-488A-A0E8-5543147B756E}"/>
   </bookViews>
   <sheets>
     <sheet name="TC-D5" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="150">
   <si>
     <t>Gallon per mile</t>
   </si>
@@ -430,6 +430,69 @@
   </si>
   <si>
     <t>CityDto</t>
+  </si>
+  <si>
+    <t>screen, pygame, car</t>
+  </si>
+  <si>
+    <t>add_destination</t>
+  </si>
+  <si>
+    <t>set_start_position</t>
+  </si>
+  <si>
+    <t>self.start_position</t>
+  </si>
+  <si>
+    <t xml:space="preserve">self.end_position </t>
+  </si>
+  <si>
+    <t>drive(self)</t>
+  </si>
+  <si>
+    <t>(250, 250)</t>
+  </si>
+  <si>
+    <t>(500, 600)</t>
+  </si>
+  <si>
+    <t>SelfDrivingCar()</t>
+  </si>
+  <si>
+    <t>create 4 potential positions</t>
+  </si>
+  <si>
+    <t>calc the distances to end_position</t>
+  </si>
+  <si>
+    <t>choose one of the positions with shortest distances (next_position)</t>
+  </si>
+  <si>
+    <t>set self.position to that  next position</t>
+  </si>
+  <si>
+    <t>show()</t>
+  </si>
+  <si>
+    <t>set self.position to start_position</t>
+  </si>
+  <si>
+    <t>self.car</t>
+  </si>
+  <si>
+    <t>create 4 potential positions ()</t>
+  </si>
+  <si>
+    <t xml:space="preserve">self.position </t>
+  </si>
+  <si>
+    <t>return a list of 4 position</t>
+  </si>
+  <si>
+    <t>calc the distance of each position for that list</t>
+  </si>
+  <si>
+    <t>Calc the distance between two positions(p1, p2)</t>
   </si>
 </sst>
 </file>
@@ -473,7 +536,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -576,11 +639,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -595,15 +682,18 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2024,7 +2114,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EED5C1B-0A68-4559-9466-4CCE32F032D5}">
-  <dimension ref="D3:T55"/>
+  <dimension ref="D3:T84"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="3" spans="6:20" x14ac:dyDescent="0.3">
@@ -2380,6 +2470,134 @@
     <row r="55" spans="4:8" x14ac:dyDescent="0.3">
       <c r="H55" t="s">
         <v>128</v>
+      </c>
+    </row>
+    <row r="58" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D58" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="59" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="F59" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="60" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="G60" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="61" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="G61" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="62" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="G62" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="63" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="F63" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="64" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="F64" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="66" spans="6:18" x14ac:dyDescent="0.3">
+      <c r="F66" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="67" spans="6:18" x14ac:dyDescent="0.3">
+      <c r="G67" t="s">
+        <v>132</v>
+      </c>
+      <c r="H67" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="68" spans="6:18" x14ac:dyDescent="0.3">
+      <c r="G68" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="70" spans="6:18" x14ac:dyDescent="0.3">
+      <c r="J70" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="71" spans="6:18" x14ac:dyDescent="0.3">
+      <c r="J71" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="72" spans="6:18" x14ac:dyDescent="0.3">
+      <c r="G72" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="73" spans="6:18" x14ac:dyDescent="0.3">
+      <c r="H73" t="s">
+        <v>139</v>
+      </c>
+      <c r="N73" s="9"/>
+      <c r="O73" s="4"/>
+      <c r="P73" s="18"/>
+      <c r="Q73" s="4"/>
+      <c r="R73" s="4"/>
+    </row>
+    <row r="74" spans="6:18" x14ac:dyDescent="0.3">
+      <c r="H74" t="s">
+        <v>140</v>
+      </c>
+      <c r="O74" s="7"/>
+      <c r="P74" s="19"/>
+      <c r="Q74" s="7"/>
+      <c r="R74" s="7"/>
+    </row>
+    <row r="75" spans="6:18" x14ac:dyDescent="0.3">
+      <c r="H75" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="76" spans="6:18" x14ac:dyDescent="0.3">
+      <c r="H76" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="77" spans="6:18" x14ac:dyDescent="0.3">
+      <c r="Q77" s="9"/>
+      <c r="R77" s="4"/>
+    </row>
+    <row r="78" spans="6:18" x14ac:dyDescent="0.3">
+      <c r="F78" t="s">
+        <v>145</v>
+      </c>
+      <c r="R78" s="7"/>
+    </row>
+    <row r="79" spans="6:18" x14ac:dyDescent="0.3">
+      <c r="G79" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="80" spans="6:18" x14ac:dyDescent="0.3">
+      <c r="G80" t="s">
+        <v>147</v>
+      </c>
+      <c r="J80" s="17"/>
+    </row>
+    <row r="82" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F82" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="84" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F84" t="s">
+        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -2736,7 +2954,7 @@
       </c>
     </row>
     <row r="3" spans="1:101" x14ac:dyDescent="0.3">
-      <c r="K3" s="16"/>
+      <c r="K3" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2754,12 +2972,12 @@
   </cols>
   <sheetData>
     <row r="10" spans="6:12" x14ac:dyDescent="0.3">
-      <c r="I10" s="14" t="s">
+      <c r="I10" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="J10" s="14"/>
-      <c r="K10" s="14"/>
-      <c r="L10" s="14"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15"/>
+      <c r="L10" s="15"/>
     </row>
     <row r="11" spans="6:12" x14ac:dyDescent="0.3">
       <c r="I11" s="1" t="s">
@@ -2776,7 +2994,7 @@
       </c>
     </row>
     <row r="12" spans="6:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F12" s="15" t="s">
+      <c r="F12" s="16" t="s">
         <v>21</v>
       </c>
       <c r="G12" s="1" t="s">
@@ -2798,7 +3016,7 @@
       </c>
     </row>
     <row r="13" spans="6:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F13" s="15"/>
+      <c r="F13" s="16"/>
       <c r="G13" s="1" t="s">
         <v>34</v>
       </c>
@@ -2818,7 +3036,7 @@
       </c>
     </row>
     <row r="14" spans="6:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F14" s="15"/>
+      <c r="F14" s="16"/>
       <c r="G14" s="1" t="s">
         <v>35</v>
       </c>
@@ -2838,7 +3056,7 @@
       </c>
     </row>
     <row r="15" spans="6:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F15" s="15"/>
+      <c r="F15" s="16"/>
       <c r="G15" s="1" t="s">
         <v>36</v>
       </c>

</xml_diff>

<commit_message>
added moving cars to pygame map
</commit_message>
<xml_diff>
--- a/unit_tests/test_cases.xlsx
+++ b/unit_tests/test_cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aa4f6975e0189fcb/Documents/Source/Cars/unit_tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="357" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{931E9543-C5CA-4AE8-BEB0-5CCB31AE1403}"/>
+  <xr:revisionPtr revIDLastSave="437" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7014EB80-35CC-45F9-954C-4C43354963DC}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="5" xr2:uid="{E1449062-40AE-488A-A0E8-5543147B756E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{E1449062-40AE-488A-A0E8-5543147B756E}"/>
   </bookViews>
   <sheets>
     <sheet name="TC-D5" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="173">
   <si>
     <t>Gallon per mile</t>
   </si>
@@ -493,13 +493,82 @@
   </si>
   <si>
     <t>Calc the distance between two positions(p1, p2)</t>
+  </si>
+  <si>
+    <t>(</t>
+  </si>
+  <si>
+    <t>(125, 85)</t>
+  </si>
+  <si>
+    <t>(115, 85)</t>
+  </si>
+  <si>
+    <t>(125,95)</t>
+  </si>
+  <si>
+    <t>(135, 85)</t>
+  </si>
+  <si>
+    <t>(125,75)</t>
+  </si>
+  <si>
+    <t>(700,85)</t>
+  </si>
+  <si>
+    <t>Position Test Cases</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#1, horizontal right </t>
+  </si>
+  <si>
+    <t>(50, 85)</t>
+  </si>
+  <si>
+    <t>(125, 50)</t>
+  </si>
+  <si>
+    <t>(125, 150)</t>
+  </si>
+  <si>
+    <t>(50, 50)</t>
+  </si>
+  <si>
+    <t>(50, 150)</t>
+  </si>
+  <si>
+    <t>(700, 150)</t>
+  </si>
+  <si>
+    <t>(700, 50)</t>
+  </si>
+  <si>
+    <t>(145, 85)</t>
+  </si>
+  <si>
+    <t>(110, 110)</t>
+  </si>
+  <si>
+    <t>(100, 100)</t>
+  </si>
+  <si>
+    <t>(110, 90)</t>
+  </si>
+  <si>
+    <t>(400, 100)</t>
+  </si>
+  <si>
+    <t>(90, 90)</t>
+  </si>
+  <si>
+    <t>(90, 110)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -515,8 +584,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -535,8 +610,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="12">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -663,11 +744,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -685,15 +779,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1502,7 +1601,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D612AEE7-2A47-4D5F-981E-E967ED3E7452}">
-  <dimension ref="F3:L26"/>
+  <dimension ref="F3:N48"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="6" max="7" width="14.109375" bestFit="1" customWidth="1"/>
@@ -1685,7 +1784,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="17" spans="6:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="6:14" x14ac:dyDescent="0.3">
       <c r="F17">
         <v>15</v>
       </c>
@@ -1693,7 +1792,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="18" spans="6:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="6:14" x14ac:dyDescent="0.3">
       <c r="F18">
         <v>15</v>
       </c>
@@ -1702,12 +1801,12 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="19" spans="6:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="6:14" x14ac:dyDescent="0.3">
       <c r="F19">
         <v>15</v>
       </c>
     </row>
-    <row r="22" spans="6:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="6:14" x14ac:dyDescent="0.3">
       <c r="F22" t="s">
         <v>11</v>
       </c>
@@ -1721,7 +1820,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="6:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="6:14" x14ac:dyDescent="0.3">
       <c r="F23" t="s">
         <v>14</v>
       </c>
@@ -1735,14 +1834,175 @@
         <v>12</v>
       </c>
     </row>
-    <row r="25" spans="6:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="6:14" x14ac:dyDescent="0.3">
       <c r="F25" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="26" spans="6:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="6:14" x14ac:dyDescent="0.3">
       <c r="F26" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="F29" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="30" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="F30" s="19" t="s">
+        <v>163</v>
+      </c>
+      <c r="I30" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="N30" s="20" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="31" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="G31" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="32" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="I32" t="s">
+        <v>153</v>
+      </c>
+      <c r="K32" s="9"/>
+      <c r="L32" s="4"/>
+    </row>
+    <row r="33" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="F33" s="19" t="s">
+        <v>159</v>
+      </c>
+      <c r="H33" t="s">
+        <v>152</v>
+      </c>
+      <c r="I33" s="19" t="s">
+        <v>151</v>
+      </c>
+      <c r="J33" t="s">
+        <v>154</v>
+      </c>
+      <c r="K33" t="s">
+        <v>166</v>
+      </c>
+      <c r="L33" s="7"/>
+      <c r="N33" s="19" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="34" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="I34" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="36" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="F36" s="19" t="s">
+        <v>162</v>
+      </c>
+      <c r="I36" s="19" t="s">
+        <v>160</v>
+      </c>
+      <c r="N36" s="19" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="41" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="F41">
+        <f>(95-85)^2</f>
+        <v>100</v>
+      </c>
+      <c r="G41">
+        <f>(75-85)^2</f>
+        <v>100</v>
+      </c>
+      <c r="H41">
+        <f>(75-85)^2</f>
+        <v>100</v>
+      </c>
+      <c r="I41">
+        <f>(95-85)^2</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="42" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="F42">
+        <f>(135-700)^2</f>
+        <v>319225</v>
+      </c>
+      <c r="G42">
+        <f>(135-700)^2</f>
+        <v>319225</v>
+      </c>
+      <c r="H42">
+        <f>(115-700)^2</f>
+        <v>342225</v>
+      </c>
+      <c r="I42">
+        <f>(115-700)^2</f>
+        <v>342225</v>
+      </c>
+    </row>
+    <row r="43" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="F43">
+        <f>SUM(F41:F42)</f>
+        <v>319325</v>
+      </c>
+      <c r="G43">
+        <f>SUM(G41:G42)</f>
+        <v>319325</v>
+      </c>
+      <c r="H43">
+        <f>SUM(H41:H42)</f>
+        <v>342325</v>
+      </c>
+      <c r="I43">
+        <f>SUM(I41:I42)</f>
+        <v>342325</v>
+      </c>
+    </row>
+    <row r="44" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="F44">
+        <f>SQRT(F43)</f>
+        <v>565.08848864580489</v>
+      </c>
+      <c r="G44">
+        <f>SQRT(G43)</f>
+        <v>565.08848864580489</v>
+      </c>
+      <c r="H44">
+        <f>SQRT(H43)</f>
+        <v>585.08546384267663</v>
+      </c>
+      <c r="I44">
+        <f>SQRT(I43)</f>
+        <v>585.08546384267663</v>
+      </c>
+    </row>
+    <row r="46" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="F46" t="s">
+        <v>172</v>
+      </c>
+      <c r="H46" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="47" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="G47" t="s">
+        <v>168</v>
+      </c>
+      <c r="K47" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="48" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="F48" t="s">
+        <v>171</v>
+      </c>
+      <c r="H48" t="s">
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -2507,12 +2767,12 @@
         <v>130</v>
       </c>
     </row>
-    <row r="66" spans="6:18" x14ac:dyDescent="0.3">
+    <row r="66" spans="6:20" x14ac:dyDescent="0.3">
       <c r="F66" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="67" spans="6:18" x14ac:dyDescent="0.3">
+    <row r="67" spans="6:20" x14ac:dyDescent="0.3">
       <c r="G67" t="s">
         <v>132</v>
       </c>
@@ -2520,75 +2780,95 @@
         <v>135</v>
       </c>
     </row>
-    <row r="68" spans="6:18" x14ac:dyDescent="0.3">
+    <row r="68" spans="6:20" x14ac:dyDescent="0.3">
       <c r="G68" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="70" spans="6:18" x14ac:dyDescent="0.3">
+    <row r="70" spans="6:20" x14ac:dyDescent="0.3">
       <c r="J70" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="71" spans="6:18" x14ac:dyDescent="0.3">
+    <row r="71" spans="6:20" x14ac:dyDescent="0.3">
       <c r="J71" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="72" spans="6:18" x14ac:dyDescent="0.3">
+    <row r="72" spans="6:20" x14ac:dyDescent="0.3">
       <c r="G72" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="73" spans="6:18" x14ac:dyDescent="0.3">
+    <row r="73" spans="6:20" x14ac:dyDescent="0.3">
       <c r="H73" t="s">
         <v>139</v>
       </c>
       <c r="N73" s="9"/>
       <c r="O73" s="4"/>
-      <c r="P73" s="18"/>
+      <c r="P73" s="16"/>
       <c r="Q73" s="4"/>
       <c r="R73" s="4"/>
     </row>
-    <row r="74" spans="6:18" x14ac:dyDescent="0.3">
+    <row r="74" spans="6:20" x14ac:dyDescent="0.3">
       <c r="H74" t="s">
         <v>140</v>
       </c>
-      <c r="O74" s="7"/>
-      <c r="P74" s="19"/>
+      <c r="O74" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="P74" s="17"/>
       <c r="Q74" s="7"/>
       <c r="R74" s="7"/>
     </row>
-    <row r="75" spans="6:18" x14ac:dyDescent="0.3">
+    <row r="75" spans="6:20" x14ac:dyDescent="0.3">
       <c r="H75" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="76" spans="6:18" x14ac:dyDescent="0.3">
+    <row r="76" spans="6:20" x14ac:dyDescent="0.3">
       <c r="H76" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="77" spans="6:18" x14ac:dyDescent="0.3">
+    <row r="77" spans="6:20" x14ac:dyDescent="0.3">
+      <c r="O77" t="s">
+        <v>153</v>
+      </c>
       <c r="Q77" s="9"/>
       <c r="R77" s="4"/>
     </row>
-    <row r="78" spans="6:18" x14ac:dyDescent="0.3">
+    <row r="78" spans="6:20" x14ac:dyDescent="0.3">
       <c r="F78" t="s">
         <v>145</v>
       </c>
+      <c r="N78" t="s">
+        <v>152</v>
+      </c>
+      <c r="O78" t="s">
+        <v>151</v>
+      </c>
+      <c r="P78" t="s">
+        <v>154</v>
+      </c>
       <c r="R78" s="7"/>
-    </row>
-    <row r="79" spans="6:18" x14ac:dyDescent="0.3">
+      <c r="T78" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="79" spans="6:20" x14ac:dyDescent="0.3">
       <c r="G79" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="80" spans="6:18" x14ac:dyDescent="0.3">
+      <c r="O79" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="80" spans="6:20" x14ac:dyDescent="0.3">
       <c r="G80" t="s">
         <v>147</v>
       </c>
-      <c r="J80" s="17"/>
+      <c r="J80" s="15"/>
     </row>
     <row r="82" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F82" t="s">
@@ -2972,12 +3252,12 @@
   </cols>
   <sheetData>
     <row r="10" spans="6:12" x14ac:dyDescent="0.3">
-      <c r="I10" s="15" t="s">
+      <c r="I10" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="J10" s="15"/>
-      <c r="K10" s="15"/>
-      <c r="L10" s="15"/>
+      <c r="J10" s="21"/>
+      <c r="K10" s="21"/>
+      <c r="L10" s="21"/>
     </row>
     <row r="11" spans="6:12" x14ac:dyDescent="0.3">
       <c r="I11" s="1" t="s">
@@ -2994,7 +3274,7 @@
       </c>
     </row>
     <row r="12" spans="6:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F12" s="16" t="s">
+      <c r="F12" s="22" t="s">
         <v>21</v>
       </c>
       <c r="G12" s="1" t="s">
@@ -3016,7 +3296,7 @@
       </c>
     </row>
     <row r="13" spans="6:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F13" s="16"/>
+      <c r="F13" s="22"/>
       <c r="G13" s="1" t="s">
         <v>34</v>
       </c>
@@ -3036,7 +3316,7 @@
       </c>
     </row>
     <row r="14" spans="6:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F14" s="16"/>
+      <c r="F14" s="22"/>
       <c r="G14" s="1" t="s">
         <v>35</v>
       </c>
@@ -3056,7 +3336,7 @@
       </c>
     </row>
     <row r="15" spans="6:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F15" s="16"/>
+      <c r="F15" s="22"/>
       <c r="G15" s="1" t="s">
         <v>36</v>
       </c>

</xml_diff>

<commit_message>
created unit tests for testing if position was on map and road
</commit_message>
<xml_diff>
--- a/unit_tests/test_cases.xlsx
+++ b/unit_tests/test_cases.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aa4f6975e0189fcb/Documents/Source/Cars/unit_tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="437" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7014EB80-35CC-45F9-954C-4C43354963DC}"/>
+  <xr:revisionPtr revIDLastSave="677" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B0CE952-0625-486C-9FAB-840B752463BA}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{E1449062-40AE-488A-A0E8-5543147B756E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="6" xr2:uid="{E1449062-40AE-488A-A0E8-5543147B756E}"/>
   </bookViews>
   <sheets>
     <sheet name="TC-D5" sheetId="1" r:id="rId1"/>
     <sheet name="TC-D2-FG-D1" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
+    <sheet name="Direction" sheetId="3" r:id="rId3"/>
     <sheet name="Design" sheetId="5" r:id="rId4"/>
     <sheet name="Database-Design" sheetId="6" r:id="rId5"/>
     <sheet name="App-Design" sheetId="7" r:id="rId6"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="231">
   <si>
     <t>Gallon per mile</t>
   </si>
@@ -562,6 +562,180 @@
   </si>
   <si>
     <t>(90, 110)</t>
+  </si>
+  <si>
+    <t>Thinking in Machine languages</t>
+  </si>
+  <si>
+    <t>Step</t>
+  </si>
+  <si>
+    <t>Machine</t>
+  </si>
+  <si>
+    <t>Position</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Array/List </t>
+  </si>
+  <si>
+    <t>arr</t>
+  </si>
+  <si>
+    <t>arr[0]</t>
+  </si>
+  <si>
+    <t>arr[1]</t>
+  </si>
+  <si>
+    <t>arr[2]</t>
+  </si>
+  <si>
+    <t>arr[3]</t>
+  </si>
+  <si>
+    <t>arr[4]</t>
+  </si>
+  <si>
+    <t>arr[5]</t>
+  </si>
+  <si>
+    <t>i = 1</t>
+  </si>
+  <si>
+    <t>j = 5</t>
+  </si>
+  <si>
+    <t>Temp = arr[i]</t>
+  </si>
+  <si>
+    <t>arr[j] = Temp</t>
+  </si>
+  <si>
+    <t>arr[i]  = arr[j]</t>
+  </si>
+  <si>
+    <t>smallest = 1,000,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">smallest = </t>
+  </si>
+  <si>
+    <t>class</t>
+  </si>
+  <si>
+    <t>find_smallest_number</t>
+  </si>
+  <si>
+    <t>find_smallest_number_position</t>
+  </si>
+  <si>
+    <t>find_largest_number</t>
+  </si>
+  <si>
+    <t>find_lasgest_number_position</t>
+  </si>
+  <si>
+    <t>swap</t>
+  </si>
+  <si>
+    <t>sort</t>
+  </si>
+  <si>
+    <t>sort_one_pass</t>
+  </si>
+  <si>
+    <t>FancyArray(self, arr)</t>
+  </si>
+  <si>
+    <t>Position (x, y)</t>
+  </si>
+  <si>
+    <t>Test pos 1</t>
+  </si>
+  <si>
+    <t>Test pos 2</t>
+  </si>
+  <si>
+    <t>test pos #3</t>
+  </si>
+  <si>
+    <t>test pos #4</t>
+  </si>
+  <si>
+    <t>test pos #5</t>
+  </si>
+  <si>
+    <t>top left (x1,y1)</t>
+  </si>
+  <si>
+    <t>top right (x2, y2)</t>
+  </si>
+  <si>
+    <t>bottom left (x3, y3)</t>
+  </si>
+  <si>
+    <t>bottom right (x4, y4)</t>
+  </si>
+  <si>
+    <t>&gt;</t>
+  </si>
+  <si>
+    <t>Destination</t>
+  </si>
+  <si>
+    <t>Picture</t>
+  </si>
+  <si>
+    <t>Dallas</t>
+  </si>
+  <si>
+    <t>Atlant</t>
+  </si>
+  <si>
+    <t>I-10</t>
+  </si>
+  <si>
+    <t>I-85</t>
+  </si>
+  <si>
+    <t>I-1</t>
+  </si>
+  <si>
+    <t>I-90</t>
+  </si>
+  <si>
+    <t>I-30</t>
+  </si>
+  <si>
+    <t>I-100</t>
+  </si>
+  <si>
+    <t>I-45</t>
+  </si>
+  <si>
+    <t>I-110</t>
+  </si>
+  <si>
+    <t>Cell Width: 50</t>
+  </si>
+  <si>
+    <t>Cell Length: 20</t>
+  </si>
+  <si>
+    <t>Length: 800</t>
+  </si>
+  <si>
+    <t>Scale Factor: 40</t>
+  </si>
+  <si>
+    <t>Scale Factor: 28.72</t>
+  </si>
+  <si>
+    <t>Width: 1536</t>
+  </si>
+  <si>
+    <t>Scale Factor: 24.7</t>
   </si>
 </sst>
 </file>
@@ -591,7 +765,7 @@
       <family val="3"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -613,6 +787,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.34998626667073579"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -761,7 +953,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -787,10 +979,20 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="3" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -811,6 +1013,231 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>69</xdr:col>
+      <xdr:colOff>185062</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>174173</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>73</xdr:col>
+      <xdr:colOff>10890</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>19481</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{20214FD6-0E06-26A9-EC50-28D11958C7E2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13705119" y="1839687"/>
+          <a:ext cx="609600" cy="585537"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>70</xdr:col>
+      <xdr:colOff>12031</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>173028</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>73</xdr:col>
+      <xdr:colOff>9739</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>42400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{12CCA4FF-8C89-4600-BDE1-3A270BE99813}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="5400000">
+          <a:off x="13716000" y="2590802"/>
+          <a:ext cx="609600" cy="585537"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>50</xdr:col>
+      <xdr:colOff>194009</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>54</xdr:col>
+      <xdr:colOff>10891</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>21772</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{23E869A7-7B08-479A-8F6B-610605EC8D16}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9991152" y="1295400"/>
+          <a:ext cx="600653" cy="576943"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>76</xdr:col>
+      <xdr:colOff>12030</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>162140</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>79</xdr:col>
+      <xdr:colOff>2118</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>31512</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9CD83AF6-B89B-4D5F-B805-DBDE0A0B4678}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="16200000">
+          <a:off x="14887846" y="2583724"/>
+          <a:ext cx="609600" cy="577917"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>76</xdr:col>
+      <xdr:colOff>10886</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>174171</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>79</xdr:col>
+      <xdr:colOff>32657</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>19479</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DDB830D1-493D-4794-88FC-C2113AB69EE9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="10800000">
+          <a:off x="14902543" y="1839685"/>
+          <a:ext cx="609600" cy="585537"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -1601,15 +2028,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D612AEE7-2A47-4D5F-981E-E967ED3E7452}">
-  <dimension ref="F3:N48"/>
+  <dimension ref="F3:Q80"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="6" max="7" width="14.109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.33203125" customWidth="1"/>
+    <col min="9" max="10" width="10.77734375" customWidth="1"/>
+    <col min="11" max="11" width="28.109375" customWidth="1"/>
+    <col min="12" max="18" width="10.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="6:12" x14ac:dyDescent="0.3">
@@ -2005,8 +2431,282 @@
         <v>169</v>
       </c>
     </row>
+    <row r="51" spans="6:17" x14ac:dyDescent="0.3">
+      <c r="F51" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="52" spans="6:17" x14ac:dyDescent="0.3">
+      <c r="J52" t="s">
+        <v>178</v>
+      </c>
+      <c r="K52" t="s">
+        <v>177</v>
+      </c>
+      <c r="L52" s="10">
+        <v>5</v>
+      </c>
+      <c r="M52" s="11">
+        <v>8</v>
+      </c>
+      <c r="N52" s="10">
+        <v>3</v>
+      </c>
+      <c r="O52" s="10">
+        <v>0</v>
+      </c>
+      <c r="P52" s="10">
+        <v>4</v>
+      </c>
+      <c r="Q52" s="21">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="53" spans="6:17" x14ac:dyDescent="0.3">
+      <c r="K53" t="s">
+        <v>176</v>
+      </c>
+      <c r="L53">
+        <v>0</v>
+      </c>
+      <c r="M53">
+        <v>1</v>
+      </c>
+      <c r="N53">
+        <v>2</v>
+      </c>
+      <c r="O53">
+        <v>3</v>
+      </c>
+      <c r="P53">
+        <v>4</v>
+      </c>
+      <c r="Q53">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="54" spans="6:17" x14ac:dyDescent="0.3">
+      <c r="L54" t="s">
+        <v>179</v>
+      </c>
+      <c r="M54" t="s">
+        <v>180</v>
+      </c>
+      <c r="N54" t="s">
+        <v>181</v>
+      </c>
+      <c r="O54" t="s">
+        <v>182</v>
+      </c>
+      <c r="P54" t="s">
+        <v>183</v>
+      </c>
+      <c r="Q54" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="56" spans="6:17" x14ac:dyDescent="0.3">
+      <c r="F56" t="s">
+        <v>175</v>
+      </c>
+      <c r="G56" t="s">
+        <v>174</v>
+      </c>
+      <c r="H56">
+        <v>1</v>
+      </c>
+      <c r="K56" t="s">
+        <v>185</v>
+      </c>
+      <c r="M56">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="6:17" x14ac:dyDescent="0.3">
+      <c r="H57">
+        <v>2</v>
+      </c>
+      <c r="K57" t="s">
+        <v>186</v>
+      </c>
+      <c r="Q57">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="58" spans="6:17" x14ac:dyDescent="0.3">
+      <c r="H58">
+        <v>3</v>
+      </c>
+      <c r="K58" t="s">
+        <v>187</v>
+      </c>
+      <c r="M58">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="59" spans="6:17" x14ac:dyDescent="0.3">
+      <c r="H59">
+        <v>4</v>
+      </c>
+      <c r="K59" t="s">
+        <v>189</v>
+      </c>
+      <c r="M59">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="60" spans="6:17" x14ac:dyDescent="0.3">
+      <c r="L60" s="10">
+        <v>5</v>
+      </c>
+      <c r="M60" s="21">
+        <v>6</v>
+      </c>
+      <c r="N60" s="10">
+        <v>3</v>
+      </c>
+      <c r="O60" s="10">
+        <v>0</v>
+      </c>
+      <c r="P60" s="10">
+        <v>4</v>
+      </c>
+      <c r="Q60" s="21">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="61" spans="6:17" x14ac:dyDescent="0.3">
+      <c r="H61">
+        <v>5</v>
+      </c>
+      <c r="K61" t="s">
+        <v>188</v>
+      </c>
+      <c r="Q61">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="62" spans="6:17" x14ac:dyDescent="0.3">
+      <c r="L62" s="10">
+        <v>5</v>
+      </c>
+      <c r="M62" s="21">
+        <v>6</v>
+      </c>
+      <c r="N62" s="10">
+        <v>3</v>
+      </c>
+      <c r="O62" s="10">
+        <v>0</v>
+      </c>
+      <c r="P62" s="10">
+        <v>4</v>
+      </c>
+      <c r="Q62" s="11">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="63" spans="6:17" x14ac:dyDescent="0.3">
+      <c r="H63">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="64" spans="6:17" x14ac:dyDescent="0.3">
+      <c r="H64">
+        <v>7</v>
+      </c>
+      <c r="K64" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="65" spans="8:11" x14ac:dyDescent="0.3">
+      <c r="H65">
+        <v>8</v>
+      </c>
+      <c r="K65" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="66" spans="8:11" x14ac:dyDescent="0.3">
+      <c r="H66">
+        <v>9</v>
+      </c>
+      <c r="K66" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="67" spans="8:11" x14ac:dyDescent="0.3">
+      <c r="H67">
+        <v>10</v>
+      </c>
+      <c r="K67" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="68" spans="8:11" x14ac:dyDescent="0.3">
+      <c r="H68">
+        <v>11</v>
+      </c>
+      <c r="K68" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="69" spans="8:11" x14ac:dyDescent="0.3">
+      <c r="K69" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="70" spans="8:11" x14ac:dyDescent="0.3">
+      <c r="K70" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="73" spans="8:11" x14ac:dyDescent="0.3">
+      <c r="H73" t="s">
+        <v>192</v>
+      </c>
+      <c r="I73" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="74" spans="8:11" x14ac:dyDescent="0.3">
+      <c r="J74" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="75" spans="8:11" x14ac:dyDescent="0.3">
+      <c r="J75" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="76" spans="8:11" x14ac:dyDescent="0.3">
+      <c r="J76" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="77" spans="8:11" x14ac:dyDescent="0.3">
+      <c r="J77" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="78" spans="8:11" x14ac:dyDescent="0.3">
+      <c r="J78" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="79" spans="8:11" x14ac:dyDescent="0.3">
+      <c r="J79" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="80" spans="8:11" x14ac:dyDescent="0.3">
+      <c r="J80" t="s">
+        <v>199</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2097,7 +2797,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46642B3E-9567-4AC5-8FF2-4527A422CDA5}">
-  <dimension ref="H3:N11"/>
+  <dimension ref="G3:N22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="9" max="9" width="12.88671875" bestFit="1" customWidth="1"/>
@@ -2158,6 +2858,60 @@
       </c>
       <c r="N11" t="s">
         <v>45</v>
+      </c>
+    </row>
+    <row r="13" spans="8:14" x14ac:dyDescent="0.3">
+      <c r="J13" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="14" spans="8:14" x14ac:dyDescent="0.3">
+      <c r="H14" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="15" spans="8:14" x14ac:dyDescent="0.3">
+      <c r="I15" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="J15" s="6"/>
+      <c r="K15" s="3" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="16" spans="8:14" x14ac:dyDescent="0.3">
+      <c r="I16" s="7"/>
+      <c r="K16" s="8"/>
+    </row>
+    <row r="17" spans="7:13" x14ac:dyDescent="0.3">
+      <c r="G17" t="s">
+        <v>202</v>
+      </c>
+      <c r="I17" s="7"/>
+      <c r="J17" t="s">
+        <v>206</v>
+      </c>
+      <c r="K17" s="8"/>
+      <c r="M17" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="18" spans="7:13" x14ac:dyDescent="0.3">
+      <c r="I18" s="7"/>
+      <c r="K18" s="8"/>
+    </row>
+    <row r="19" spans="7:13" x14ac:dyDescent="0.3">
+      <c r="I19" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="J19" s="9"/>
+      <c r="K19" s="5" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="22" spans="7:13" x14ac:dyDescent="0.3">
+      <c r="J22" t="s">
+        <v>205</v>
       </c>
     </row>
   </sheetData>
@@ -2887,7 +3641,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B4D1224-06E7-451A-AAFD-053F2614A910}">
-  <dimension ref="A1:CW3"/>
+  <dimension ref="A1:CW26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="144" width="2.77734375" customWidth="1"/>
@@ -3236,8 +3990,297 @@
     <row r="3" spans="1:101" x14ac:dyDescent="0.3">
       <c r="K3" s="14"/>
     </row>
+    <row r="5" spans="1:101" x14ac:dyDescent="0.3">
+      <c r="BF5" t="s">
+        <v>223</v>
+      </c>
+      <c r="BI5" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="6" spans="1:101" x14ac:dyDescent="0.3">
+      <c r="N6" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="7" spans="1:101" x14ac:dyDescent="0.3">
+      <c r="L7" s="24"/>
+      <c r="M7" s="25"/>
+      <c r="N7" s="25"/>
+      <c r="O7" s="25"/>
+      <c r="AB7" t="s">
+        <v>219</v>
+      </c>
+      <c r="AP7" s="26"/>
+      <c r="AQ7" s="26"/>
+      <c r="AR7" s="26"/>
+      <c r="AS7" s="26"/>
+      <c r="BD7" s="25"/>
+      <c r="BE7" s="25"/>
+      <c r="BF7" s="25"/>
+      <c r="BG7" s="25"/>
+      <c r="BH7" s="25"/>
+      <c r="BI7" s="24"/>
+    </row>
+    <row r="8" spans="1:101" x14ac:dyDescent="0.3">
+      <c r="J8" t="s">
+        <v>91</v>
+      </c>
+      <c r="O8" s="25"/>
+      <c r="AP8" s="26"/>
+      <c r="AQ8" s="26"/>
+      <c r="AR8" s="26"/>
+      <c r="AS8" s="26"/>
+      <c r="BD8" s="25"/>
+    </row>
+    <row r="9" spans="1:101" x14ac:dyDescent="0.3">
+      <c r="O9" s="25"/>
+      <c r="P9" s="25"/>
+      <c r="Q9" s="25"/>
+      <c r="R9" s="25"/>
+      <c r="S9" s="25"/>
+      <c r="T9" s="25"/>
+      <c r="U9" s="25"/>
+      <c r="V9" s="25"/>
+      <c r="W9" s="25"/>
+      <c r="X9" s="25"/>
+      <c r="Y9" s="25"/>
+      <c r="Z9" s="25"/>
+      <c r="AA9" s="25"/>
+      <c r="AB9" s="25"/>
+      <c r="AC9" s="25"/>
+      <c r="AD9" s="25"/>
+      <c r="AE9" s="25"/>
+      <c r="AF9" s="25"/>
+      <c r="AG9" s="25"/>
+      <c r="AH9" s="25"/>
+      <c r="AI9" s="25"/>
+      <c r="AJ9" s="25"/>
+      <c r="AK9" s="25"/>
+      <c r="AL9" s="25"/>
+      <c r="AM9" s="25"/>
+      <c r="AN9" s="24"/>
+      <c r="AO9" s="25"/>
+      <c r="AP9" s="25"/>
+      <c r="AQ9" s="25"/>
+      <c r="AR9" s="29"/>
+      <c r="AS9" s="25"/>
+      <c r="AT9" s="25"/>
+      <c r="AU9" s="25"/>
+      <c r="AV9" s="25"/>
+      <c r="AW9" s="25"/>
+      <c r="AX9" s="25"/>
+      <c r="AY9" s="25"/>
+      <c r="AZ9" s="25"/>
+      <c r="BA9" s="25"/>
+      <c r="BB9" s="25"/>
+      <c r="BC9" s="25"/>
+      <c r="BD9" s="25"/>
+      <c r="BS9" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="10" spans="1:101" x14ac:dyDescent="0.3">
+      <c r="O10" s="25"/>
+      <c r="AP10" s="26"/>
+      <c r="AQ10" s="26"/>
+      <c r="AR10" s="26"/>
+      <c r="AS10" s="26"/>
+      <c r="AU10" s="26"/>
+      <c r="AV10" s="26"/>
+      <c r="BD10" s="25"/>
+    </row>
+    <row r="11" spans="1:101" x14ac:dyDescent="0.3">
+      <c r="O11" s="25"/>
+      <c r="AP11" s="26"/>
+      <c r="AQ11" s="26"/>
+      <c r="AR11" s="26"/>
+      <c r="AS11" s="26"/>
+      <c r="BD11" s="25"/>
+      <c r="BM11" s="28"/>
+    </row>
+    <row r="12" spans="1:101" x14ac:dyDescent="0.3">
+      <c r="M12" t="s">
+        <v>218</v>
+      </c>
+      <c r="O12" s="25"/>
+      <c r="BD12" s="25"/>
+      <c r="BL12" s="28"/>
+      <c r="BM12" s="30" t="s">
+        <v>211</v>
+      </c>
+      <c r="BN12" s="28"/>
+    </row>
+    <row r="13" spans="1:101" x14ac:dyDescent="0.3">
+      <c r="O13" s="25"/>
+      <c r="BD13" s="25"/>
+      <c r="BM13" s="28"/>
+    </row>
+    <row r="14" spans="1:101" x14ac:dyDescent="0.3">
+      <c r="O14" s="25"/>
+      <c r="BD14" s="25"/>
+    </row>
+    <row r="15" spans="1:101" x14ac:dyDescent="0.3">
+      <c r="O15" s="25"/>
+      <c r="BD15" s="25"/>
+      <c r="BF15" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="16" spans="1:101" x14ac:dyDescent="0.3">
+      <c r="O16" s="25"/>
+      <c r="BD16" s="25"/>
+    </row>
+    <row r="17" spans="14:77" x14ac:dyDescent="0.3">
+      <c r="O17" s="25"/>
+      <c r="BD17" s="25"/>
+    </row>
+    <row r="18" spans="14:77" x14ac:dyDescent="0.3">
+      <c r="O18" s="24"/>
+      <c r="P18" s="25"/>
+      <c r="Q18" s="25"/>
+      <c r="R18" s="25"/>
+      <c r="S18" s="25"/>
+      <c r="T18" s="25"/>
+      <c r="U18" s="25"/>
+      <c r="V18" s="25"/>
+      <c r="W18" s="25"/>
+      <c r="X18" s="25"/>
+      <c r="Y18" s="25"/>
+      <c r="Z18" s="25"/>
+      <c r="AA18" s="25"/>
+      <c r="AB18" s="25"/>
+      <c r="AC18" s="25"/>
+      <c r="AD18" s="25"/>
+      <c r="AE18" s="25"/>
+      <c r="AF18" s="25"/>
+      <c r="BD18" s="25"/>
+    </row>
+    <row r="19" spans="14:77" x14ac:dyDescent="0.3">
+      <c r="AF19" s="25"/>
+      <c r="BD19" s="25"/>
+      <c r="BK19" s="26"/>
+      <c r="BL19" s="26"/>
+      <c r="BM19" s="26"/>
+      <c r="BN19" s="26" t="s">
+        <v>229</v>
+      </c>
+      <c r="BO19" s="26"/>
+      <c r="BP19" s="26"/>
+      <c r="BQ19" s="26"/>
+    </row>
+    <row r="20" spans="14:77" x14ac:dyDescent="0.3">
+      <c r="N20" t="s">
+        <v>92</v>
+      </c>
+      <c r="W20" t="s">
+        <v>220</v>
+      </c>
+      <c r="AF20" s="25"/>
+      <c r="BD20" s="25"/>
+      <c r="BK20" s="26"/>
+      <c r="BL20" s="26"/>
+      <c r="BM20" s="26"/>
+      <c r="BN20" s="26" t="s">
+        <v>226</v>
+      </c>
+      <c r="BO20" s="26"/>
+      <c r="BP20" s="26"/>
+      <c r="BQ20" s="26"/>
+    </row>
+    <row r="21" spans="14:77" x14ac:dyDescent="0.3">
+      <c r="AD21" t="s">
+        <v>222</v>
+      </c>
+      <c r="AF21" s="25"/>
+      <c r="BD21" s="25"/>
+      <c r="BK21" s="26"/>
+      <c r="BL21" s="26"/>
+      <c r="BM21" s="27"/>
+      <c r="BN21" s="26"/>
+      <c r="BO21" s="26"/>
+      <c r="BP21" s="26"/>
+      <c r="BQ21" s="26"/>
+    </row>
+    <row r="22" spans="14:77" x14ac:dyDescent="0.3">
+      <c r="AF22" s="25"/>
+      <c r="AG22" s="25"/>
+      <c r="AH22" s="25"/>
+      <c r="AI22" s="25"/>
+      <c r="AJ22" s="25"/>
+      <c r="AK22" s="25"/>
+      <c r="AL22" s="25"/>
+      <c r="AM22" s="25"/>
+      <c r="AN22" s="25"/>
+      <c r="AO22" s="25"/>
+      <c r="AP22" s="25"/>
+      <c r="AQ22" s="25"/>
+      <c r="AR22" s="25"/>
+      <c r="AS22" s="25"/>
+      <c r="AT22" s="25"/>
+      <c r="AU22" s="25"/>
+      <c r="AV22" s="25"/>
+      <c r="AW22" s="25"/>
+      <c r="AX22" s="25"/>
+      <c r="AY22" s="25"/>
+      <c r="AZ22" s="25"/>
+      <c r="BA22" s="25"/>
+      <c r="BB22" s="25"/>
+      <c r="BC22" s="25"/>
+      <c r="BD22" s="24"/>
+      <c r="BK22" s="26"/>
+      <c r="BL22" s="26"/>
+      <c r="BM22" s="26"/>
+      <c r="BN22" s="26" t="s">
+        <v>224</v>
+      </c>
+      <c r="BO22" s="26"/>
+      <c r="BP22" s="26"/>
+      <c r="BQ22" s="26"/>
+      <c r="BS22" t="s">
+        <v>228</v>
+      </c>
+      <c r="BY22" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="23" spans="14:77" x14ac:dyDescent="0.3">
+      <c r="AF23" s="25"/>
+      <c r="AQ23" t="s">
+        <v>216</v>
+      </c>
+      <c r="BE23" t="s">
+        <v>212</v>
+      </c>
+      <c r="BK23" s="26"/>
+      <c r="BL23" s="26"/>
+      <c r="BM23" s="26"/>
+      <c r="BN23" s="26" t="s">
+        <v>225</v>
+      </c>
+      <c r="BO23" s="26"/>
+      <c r="BP23" s="26"/>
+      <c r="BQ23" s="26"/>
+      <c r="BS23" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="24" spans="14:77" x14ac:dyDescent="0.3">
+      <c r="AF24" s="24"/>
+    </row>
+    <row r="25" spans="14:77" x14ac:dyDescent="0.3">
+      <c r="BD25" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="26" spans="14:77" x14ac:dyDescent="0.3">
+      <c r="AE26" t="s">
+        <v>214</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3252,12 +4295,12 @@
   </cols>
   <sheetData>
     <row r="10" spans="6:12" x14ac:dyDescent="0.3">
-      <c r="I10" s="21" t="s">
+      <c r="I10" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="J10" s="21"/>
-      <c r="K10" s="21"/>
-      <c r="L10" s="21"/>
+      <c r="J10" s="22"/>
+      <c r="K10" s="22"/>
+      <c r="L10" s="22"/>
     </row>
     <row r="11" spans="6:12" x14ac:dyDescent="0.3">
       <c r="I11" s="1" t="s">
@@ -3274,7 +4317,7 @@
       </c>
     </row>
     <row r="12" spans="6:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F12" s="22" t="s">
+      <c r="F12" s="23" t="s">
         <v>21</v>
       </c>
       <c r="G12" s="1" t="s">
@@ -3296,7 +4339,7 @@
       </c>
     </row>
     <row r="13" spans="6:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F13" s="22"/>
+      <c r="F13" s="23"/>
       <c r="G13" s="1" t="s">
         <v>34</v>
       </c>
@@ -3316,7 +4359,7 @@
       </c>
     </row>
     <row r="14" spans="6:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F14" s="22"/>
+      <c r="F14" s="23"/>
       <c r="G14" s="1" t="s">
         <v>35</v>
       </c>
@@ -3336,7 +4379,7 @@
       </c>
     </row>
     <row r="15" spans="6:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F15" s="22"/>
+      <c r="F15" s="23"/>
       <c r="G15" s="1" t="s">
         <v>36</v>
       </c>

</xml_diff>

<commit_message>
added new cars and modified traveling journey coding for beta testing
</commit_message>
<xml_diff>
--- a/unit_tests/test_cases.xlsx
+++ b/unit_tests/test_cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aa4f6975e0189fcb/Documents/Source/Cars/unit_tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="677" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B0CE952-0625-486C-9FAB-840B752463BA}"/>
+  <xr:revisionPtr revIDLastSave="723" documentId="8_{EBE1DB55-C704-4BE3-A773-BFD4AD0C5B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15AD4ED5-83A4-4204-A613-F745EF7D7FCF}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="6" xr2:uid="{E1449062-40AE-488A-A0E8-5543147B756E}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="244">
   <si>
     <t>Gallon per mile</t>
   </si>
@@ -736,6 +736,45 @@
   </si>
   <si>
     <t>Scale Factor: 24.7</t>
+  </si>
+  <si>
+    <t>Chicago</t>
+  </si>
+  <si>
+    <t>(201,41)</t>
+  </si>
+  <si>
+    <t>(219,498</t>
+  </si>
+  <si>
+    <t>(201,498</t>
+  </si>
+  <si>
+    <t>(235,516</t>
+  </si>
+  <si>
+    <t>x,y</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>x - W/2, y + L / 2</t>
+  </si>
+  <si>
+    <t>x - W/2, y - L/2</t>
+  </si>
+  <si>
+    <t>x + W/2, y  + L/2</t>
+  </si>
+  <si>
+    <t>x + W/2, y  - L/2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x,y = </t>
   </si>
 </sst>
 </file>
@@ -765,7 +804,7 @@
       <family val="3"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -805,6 +844,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.34998626667073579"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -953,7 +998,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -980,21 +1025,22 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="3" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1104,16 +1150,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>50</xdr:col>
-      <xdr:colOff>194009</xdr:colOff>
+      <xdr:col>51</xdr:col>
+      <xdr:colOff>9847</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>54</xdr:col>
-      <xdr:colOff>10891</xdr:colOff>
+      <xdr:colOff>5</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>21772</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1136,8 +1182,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9991152" y="1295400"/>
-          <a:ext cx="600653" cy="576943"/>
+          <a:off x="10002933" y="1295400"/>
+          <a:ext cx="577986" cy="555171"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3641,7 +3687,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B4D1224-06E7-451A-AAFD-053F2614A910}">
-  <dimension ref="A1:CW26"/>
+  <dimension ref="A1:CW38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="144" width="2.77734375" customWidth="1"/>
@@ -4004,170 +4050,149 @@
       </c>
     </row>
     <row r="7" spans="1:101" x14ac:dyDescent="0.3">
-      <c r="L7" s="24"/>
-      <c r="M7" s="25"/>
-      <c r="N7" s="25"/>
-      <c r="O7" s="25"/>
+      <c r="L7" s="22"/>
+      <c r="M7" s="23"/>
+      <c r="N7" s="23"/>
+      <c r="O7" s="23"/>
       <c r="AB7" t="s">
         <v>219</v>
       </c>
-      <c r="AP7" s="26"/>
-      <c r="AQ7" s="26"/>
-      <c r="AR7" s="26"/>
-      <c r="AS7" s="26"/>
-      <c r="BD7" s="25"/>
-      <c r="BE7" s="25"/>
-      <c r="BF7" s="25"/>
-      <c r="BG7" s="25"/>
-      <c r="BH7" s="25"/>
-      <c r="BI7" s="24"/>
+      <c r="BD7" s="23"/>
+      <c r="BE7" s="23"/>
+      <c r="BF7" s="23"/>
+      <c r="BG7" s="23"/>
+      <c r="BH7" s="23"/>
+      <c r="BI7" s="22"/>
     </row>
     <row r="8" spans="1:101" x14ac:dyDescent="0.3">
       <c r="J8" t="s">
         <v>91</v>
       </c>
-      <c r="O8" s="25"/>
-      <c r="AP8" s="26"/>
-      <c r="AQ8" s="26"/>
-      <c r="AR8" s="26"/>
-      <c r="AS8" s="26"/>
-      <c r="BD8" s="25"/>
+      <c r="O8" s="23"/>
+      <c r="BD8" s="23"/>
     </row>
     <row r="9" spans="1:101" x14ac:dyDescent="0.3">
-      <c r="O9" s="25"/>
-      <c r="P9" s="25"/>
-      <c r="Q9" s="25"/>
-      <c r="R9" s="25"/>
-      <c r="S9" s="25"/>
-      <c r="T9" s="25"/>
-      <c r="U9" s="25"/>
-      <c r="V9" s="25"/>
-      <c r="W9" s="25"/>
-      <c r="X9" s="25"/>
-      <c r="Y9" s="25"/>
-      <c r="Z9" s="25"/>
-      <c r="AA9" s="25"/>
-      <c r="AB9" s="25"/>
-      <c r="AC9" s="25"/>
-      <c r="AD9" s="25"/>
-      <c r="AE9" s="25"/>
-      <c r="AF9" s="25"/>
-      <c r="AG9" s="25"/>
-      <c r="AH9" s="25"/>
-      <c r="AI9" s="25"/>
-      <c r="AJ9" s="25"/>
-      <c r="AK9" s="25"/>
-      <c r="AL9" s="25"/>
-      <c r="AM9" s="25"/>
-      <c r="AN9" s="24"/>
-      <c r="AO9" s="25"/>
-      <c r="AP9" s="25"/>
-      <c r="AQ9" s="25"/>
-      <c r="AR9" s="29"/>
-      <c r="AS9" s="25"/>
-      <c r="AT9" s="25"/>
-      <c r="AU9" s="25"/>
-      <c r="AV9" s="25"/>
-      <c r="AW9" s="25"/>
-      <c r="AX9" s="25"/>
-      <c r="AY9" s="25"/>
-      <c r="AZ9" s="25"/>
-      <c r="BA9" s="25"/>
-      <c r="BB9" s="25"/>
-      <c r="BC9" s="25"/>
-      <c r="BD9" s="25"/>
+      <c r="O9" s="23"/>
+      <c r="P9" s="23"/>
+      <c r="Q9" s="23"/>
+      <c r="R9" s="23"/>
+      <c r="S9" s="23"/>
+      <c r="T9" s="23"/>
+      <c r="U9" s="23"/>
+      <c r="V9" s="23"/>
+      <c r="W9" s="23"/>
+      <c r="X9" s="23"/>
+      <c r="Y9" s="23"/>
+      <c r="Z9" s="23"/>
+      <c r="AA9" s="23"/>
+      <c r="AB9" s="23"/>
+      <c r="AC9" s="23"/>
+      <c r="AD9" s="23"/>
+      <c r="AE9" s="23"/>
+      <c r="AF9" s="23"/>
+      <c r="AG9" s="23"/>
+      <c r="AH9" s="23"/>
+      <c r="AI9" s="23"/>
+      <c r="AJ9" s="23"/>
+      <c r="AK9" s="23"/>
+      <c r="AL9" s="23"/>
+      <c r="AM9" s="23"/>
+      <c r="AN9" s="22"/>
+      <c r="AO9" s="23"/>
+      <c r="AP9" s="23"/>
+      <c r="AQ9" s="23"/>
+      <c r="AR9" s="25"/>
+      <c r="AS9" s="23"/>
+      <c r="AT9" s="23"/>
+      <c r="AU9" s="23"/>
+      <c r="AV9" s="23"/>
+      <c r="AW9" s="23"/>
+      <c r="AX9" s="23"/>
+      <c r="AY9" s="23"/>
+      <c r="AZ9" s="23"/>
+      <c r="BA9" s="23"/>
+      <c r="BB9" s="23"/>
+      <c r="BC9" s="23"/>
+      <c r="BD9" s="23"/>
       <c r="BS9" s="1" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="10" spans="1:101" x14ac:dyDescent="0.3">
-      <c r="O10" s="25"/>
-      <c r="AP10" s="26"/>
-      <c r="AQ10" s="26"/>
-      <c r="AR10" s="26"/>
-      <c r="AS10" s="26"/>
-      <c r="AU10" s="26"/>
-      <c r="AV10" s="26"/>
-      <c r="BD10" s="25"/>
+      <c r="O10" s="23"/>
+      <c r="AM10" t="s">
+        <v>231</v>
+      </c>
+      <c r="BD10" s="23"/>
     </row>
     <row r="11" spans="1:101" x14ac:dyDescent="0.3">
-      <c r="O11" s="25"/>
-      <c r="AP11" s="26"/>
-      <c r="AQ11" s="26"/>
-      <c r="AR11" s="26"/>
-      <c r="AS11" s="26"/>
-      <c r="BD11" s="25"/>
-      <c r="BM11" s="28"/>
+      <c r="O11" s="23"/>
+      <c r="BD11" s="23"/>
+      <c r="BM11" s="24"/>
     </row>
     <row r="12" spans="1:101" x14ac:dyDescent="0.3">
       <c r="M12" t="s">
         <v>218</v>
       </c>
-      <c r="O12" s="25"/>
-      <c r="BD12" s="25"/>
-      <c r="BL12" s="28"/>
-      <c r="BM12" s="30" t="s">
+      <c r="O12" s="23"/>
+      <c r="BD12" s="23"/>
+      <c r="BL12" s="24"/>
+      <c r="BM12" s="26" t="s">
         <v>211</v>
       </c>
-      <c r="BN12" s="28"/>
+      <c r="BN12" s="24"/>
     </row>
     <row r="13" spans="1:101" x14ac:dyDescent="0.3">
-      <c r="O13" s="25"/>
-      <c r="BD13" s="25"/>
-      <c r="BM13" s="28"/>
+      <c r="O13" s="23"/>
+      <c r="BD13" s="23"/>
+      <c r="BM13" s="24"/>
     </row>
     <row r="14" spans="1:101" x14ac:dyDescent="0.3">
-      <c r="O14" s="25"/>
-      <c r="BD14" s="25"/>
+      <c r="O14" s="23"/>
+      <c r="BD14" s="23"/>
     </row>
     <row r="15" spans="1:101" x14ac:dyDescent="0.3">
-      <c r="O15" s="25"/>
-      <c r="BD15" s="25"/>
+      <c r="O15" s="23"/>
+      <c r="BD15" s="23"/>
       <c r="BF15" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="16" spans="1:101" x14ac:dyDescent="0.3">
-      <c r="O16" s="25"/>
-      <c r="BD16" s="25"/>
+      <c r="O16" s="23"/>
+      <c r="BD16" s="23"/>
     </row>
     <row r="17" spans="14:77" x14ac:dyDescent="0.3">
-      <c r="O17" s="25"/>
-      <c r="BD17" s="25"/>
+      <c r="O17" s="23"/>
+      <c r="BD17" s="23"/>
     </row>
     <row r="18" spans="14:77" x14ac:dyDescent="0.3">
-      <c r="O18" s="24"/>
-      <c r="P18" s="25"/>
-      <c r="Q18" s="25"/>
-      <c r="R18" s="25"/>
-      <c r="S18" s="25"/>
-      <c r="T18" s="25"/>
-      <c r="U18" s="25"/>
-      <c r="V18" s="25"/>
-      <c r="W18" s="25"/>
-      <c r="X18" s="25"/>
-      <c r="Y18" s="25"/>
-      <c r="Z18" s="25"/>
-      <c r="AA18" s="25"/>
-      <c r="AB18" s="25"/>
-      <c r="AC18" s="25"/>
-      <c r="AD18" s="25"/>
-      <c r="AE18" s="25"/>
-      <c r="AF18" s="25"/>
-      <c r="BD18" s="25"/>
+      <c r="O18" s="22"/>
+      <c r="P18" s="23"/>
+      <c r="Q18" s="23"/>
+      <c r="R18" s="23"/>
+      <c r="S18" s="23"/>
+      <c r="T18" s="23"/>
+      <c r="U18" s="23"/>
+      <c r="V18" s="23"/>
+      <c r="W18" s="23"/>
+      <c r="X18" s="23"/>
+      <c r="Y18" s="23"/>
+      <c r="Z18" s="23"/>
+      <c r="AA18" s="23"/>
+      <c r="AB18" s="23"/>
+      <c r="AC18" s="23"/>
+      <c r="AD18" s="23"/>
+      <c r="AE18" s="23"/>
+      <c r="AF18" s="23"/>
+      <c r="BD18" s="23"/>
     </row>
     <row r="19" spans="14:77" x14ac:dyDescent="0.3">
-      <c r="AF19" s="25"/>
-      <c r="BD19" s="25"/>
-      <c r="BK19" s="26"/>
-      <c r="BL19" s="26"/>
-      <c r="BM19" s="26"/>
-      <c r="BN19" s="26" t="s">
+      <c r="AF19" s="23"/>
+      <c r="BD19" s="23"/>
+      <c r="BN19" t="s">
         <v>229</v>
       </c>
-      <c r="BO19" s="26"/>
-      <c r="BP19" s="26"/>
-      <c r="BQ19" s="26"/>
     </row>
     <row r="20" spans="14:77" x14ac:dyDescent="0.3">
       <c r="N20" t="s">
@@ -4176,67 +4201,49 @@
       <c r="W20" t="s">
         <v>220</v>
       </c>
-      <c r="AF20" s="25"/>
-      <c r="BD20" s="25"/>
-      <c r="BK20" s="26"/>
-      <c r="BL20" s="26"/>
-      <c r="BM20" s="26"/>
-      <c r="BN20" s="26" t="s">
+      <c r="AF20" s="23"/>
+      <c r="BD20" s="23"/>
+      <c r="BN20" t="s">
         <v>226</v>
       </c>
-      <c r="BO20" s="26"/>
-      <c r="BP20" s="26"/>
-      <c r="BQ20" s="26"/>
     </row>
     <row r="21" spans="14:77" x14ac:dyDescent="0.3">
       <c r="AD21" t="s">
         <v>222</v>
       </c>
-      <c r="AF21" s="25"/>
-      <c r="BD21" s="25"/>
-      <c r="BK21" s="26"/>
-      <c r="BL21" s="26"/>
-      <c r="BM21" s="27"/>
-      <c r="BN21" s="26"/>
-      <c r="BO21" s="26"/>
-      <c r="BP21" s="26"/>
-      <c r="BQ21" s="26"/>
+      <c r="AF21" s="23"/>
+      <c r="BD21" s="23"/>
+      <c r="BM21" s="15"/>
     </row>
     <row r="22" spans="14:77" x14ac:dyDescent="0.3">
-      <c r="AF22" s="25"/>
-      <c r="AG22" s="25"/>
-      <c r="AH22" s="25"/>
-      <c r="AI22" s="25"/>
-      <c r="AJ22" s="25"/>
-      <c r="AK22" s="25"/>
-      <c r="AL22" s="25"/>
-      <c r="AM22" s="25"/>
-      <c r="AN22" s="25"/>
-      <c r="AO22" s="25"/>
-      <c r="AP22" s="25"/>
-      <c r="AQ22" s="25"/>
-      <c r="AR22" s="25"/>
-      <c r="AS22" s="25"/>
-      <c r="AT22" s="25"/>
-      <c r="AU22" s="25"/>
-      <c r="AV22" s="25"/>
-      <c r="AW22" s="25"/>
-      <c r="AX22" s="25"/>
-      <c r="AY22" s="25"/>
-      <c r="AZ22" s="25"/>
-      <c r="BA22" s="25"/>
-      <c r="BB22" s="25"/>
-      <c r="BC22" s="25"/>
-      <c r="BD22" s="24"/>
-      <c r="BK22" s="26"/>
-      <c r="BL22" s="26"/>
-      <c r="BM22" s="26"/>
-      <c r="BN22" s="26" t="s">
+      <c r="AF22" s="23"/>
+      <c r="AG22" s="23"/>
+      <c r="AH22" s="23"/>
+      <c r="AI22" s="23"/>
+      <c r="AJ22" s="23"/>
+      <c r="AK22" s="23"/>
+      <c r="AL22" s="23"/>
+      <c r="AM22" s="23"/>
+      <c r="AN22" s="23"/>
+      <c r="AO22" s="23"/>
+      <c r="AP22" s="23"/>
+      <c r="AQ22" s="23"/>
+      <c r="AR22" s="23"/>
+      <c r="AS22" s="23"/>
+      <c r="AT22" s="23"/>
+      <c r="AU22" s="23"/>
+      <c r="AV22" s="23"/>
+      <c r="AW22" s="23"/>
+      <c r="AX22" s="23"/>
+      <c r="AY22" s="23"/>
+      <c r="AZ22" s="23"/>
+      <c r="BA22" s="23"/>
+      <c r="BB22" s="23"/>
+      <c r="BC22" s="23"/>
+      <c r="BD22" s="22"/>
+      <c r="BN22" t="s">
         <v>224</v>
       </c>
-      <c r="BO22" s="26"/>
-      <c r="BP22" s="26"/>
-      <c r="BQ22" s="26"/>
       <c r="BS22" t="s">
         <v>228</v>
       </c>
@@ -4245,28 +4252,22 @@
       </c>
     </row>
     <row r="23" spans="14:77" x14ac:dyDescent="0.3">
-      <c r="AF23" s="25"/>
+      <c r="AF23" s="23"/>
       <c r="AQ23" t="s">
         <v>216</v>
       </c>
       <c r="BE23" t="s">
         <v>212</v>
       </c>
-      <c r="BK23" s="26"/>
-      <c r="BL23" s="26"/>
-      <c r="BM23" s="26"/>
-      <c r="BN23" s="26" t="s">
+      <c r="BN23" t="s">
         <v>225</v>
       </c>
-      <c r="BO23" s="26"/>
-      <c r="BP23" s="26"/>
-      <c r="BQ23" s="26"/>
       <c r="BS23" t="s">
         <v>227</v>
       </c>
     </row>
     <row r="24" spans="14:77" x14ac:dyDescent="0.3">
-      <c r="AF24" s="24"/>
+      <c r="AF24" s="22"/>
     </row>
     <row r="25" spans="14:77" x14ac:dyDescent="0.3">
       <c r="BD25" t="s">
@@ -4277,6 +4278,107 @@
       <c r="AE26" t="s">
         <v>214</v>
       </c>
+      <c r="BE26" t="s">
+        <v>239</v>
+      </c>
+      <c r="BJ26" s="27"/>
+      <c r="BO26" s="14" t="s">
+        <v>241</v>
+      </c>
+      <c r="BP26" s="31"/>
+      <c r="BR26" s="7" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="27" spans="14:77" x14ac:dyDescent="0.3">
+      <c r="AK27" s="28"/>
+      <c r="BJ27" s="27"/>
+      <c r="BR27" s="7"/>
+    </row>
+    <row r="28" spans="14:77" x14ac:dyDescent="0.3">
+      <c r="AK28" t="s">
+        <v>232</v>
+      </c>
+      <c r="AN28" s="28"/>
+      <c r="AO28" t="s">
+        <v>234</v>
+      </c>
+      <c r="BJ28" s="27"/>
+      <c r="BR28" s="7"/>
+    </row>
+    <row r="29" spans="14:77" x14ac:dyDescent="0.3">
+      <c r="AK29" s="28" t="s">
+        <v>233</v>
+      </c>
+      <c r="AO29" t="s">
+        <v>235</v>
+      </c>
+      <c r="BJ29" s="27"/>
+      <c r="BR29" s="7"/>
+    </row>
+    <row r="30" spans="14:77" x14ac:dyDescent="0.3">
+      <c r="BJ30" s="27"/>
+      <c r="BR30" s="7"/>
+    </row>
+    <row r="31" spans="14:77" x14ac:dyDescent="0.3">
+      <c r="AK31" t="s">
+        <v>243</v>
+      </c>
+      <c r="BE31" s="27"/>
+      <c r="BF31" s="27"/>
+      <c r="BG31" s="27"/>
+      <c r="BH31" s="27"/>
+      <c r="BI31" s="27"/>
+      <c r="BJ31" t="s">
+        <v>236</v>
+      </c>
+      <c r="BK31" s="27"/>
+      <c r="BL31" s="27"/>
+      <c r="BM31" s="27"/>
+      <c r="BN31" s="27"/>
+      <c r="BO31" s="27"/>
+      <c r="BR31" s="7"/>
+    </row>
+    <row r="32" spans="14:77" x14ac:dyDescent="0.3">
+      <c r="BJ32" s="27"/>
+      <c r="BR32" s="7"/>
+    </row>
+    <row r="33" spans="57:70" x14ac:dyDescent="0.3">
+      <c r="BJ33" s="27"/>
+      <c r="BR33" s="7"/>
+    </row>
+    <row r="34" spans="57:70" x14ac:dyDescent="0.3">
+      <c r="BJ34" s="27"/>
+      <c r="BR34" s="7"/>
+    </row>
+    <row r="35" spans="57:70" x14ac:dyDescent="0.3">
+      <c r="BJ35" s="27"/>
+      <c r="BR35" s="7"/>
+    </row>
+    <row r="36" spans="57:70" x14ac:dyDescent="0.3">
+      <c r="BE36" t="s">
+        <v>240</v>
+      </c>
+      <c r="BJ36" s="27"/>
+      <c r="BO36" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="BR36" s="7"/>
+    </row>
+    <row r="38" spans="57:70" x14ac:dyDescent="0.3">
+      <c r="BE38" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="BF38" s="6"/>
+      <c r="BG38" s="6"/>
+      <c r="BH38" s="6"/>
+      <c r="BI38" s="6"/>
+      <c r="BJ38" s="6"/>
+      <c r="BK38" s="6"/>
+      <c r="BL38" s="6"/>
+      <c r="BM38" s="6"/>
+      <c r="BN38" s="6"/>
+      <c r="BO38" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4295,12 +4397,12 @@
   </cols>
   <sheetData>
     <row r="10" spans="6:12" x14ac:dyDescent="0.3">
-      <c r="I10" s="22" t="s">
+      <c r="I10" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="J10" s="22"/>
-      <c r="K10" s="22"/>
-      <c r="L10" s="22"/>
+      <c r="J10" s="29"/>
+      <c r="K10" s="29"/>
+      <c r="L10" s="29"/>
     </row>
     <row r="11" spans="6:12" x14ac:dyDescent="0.3">
       <c r="I11" s="1" t="s">
@@ -4317,7 +4419,7 @@
       </c>
     </row>
     <row r="12" spans="6:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F12" s="23" t="s">
+      <c r="F12" s="30" t="s">
         <v>21</v>
       </c>
       <c r="G12" s="1" t="s">
@@ -4339,7 +4441,7 @@
       </c>
     </row>
     <row r="13" spans="6:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F13" s="23"/>
+      <c r="F13" s="30"/>
       <c r="G13" s="1" t="s">
         <v>34</v>
       </c>
@@ -4359,7 +4461,7 @@
       </c>
     </row>
     <row r="14" spans="6:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F14" s="23"/>
+      <c r="F14" s="30"/>
       <c r="G14" s="1" t="s">
         <v>35</v>
       </c>
@@ -4379,7 +4481,7 @@
       </c>
     </row>
     <row r="15" spans="6:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F15" s="23"/>
+      <c r="F15" s="30"/>
       <c r="G15" s="1" t="s">
         <v>36</v>
       </c>

</xml_diff>